<commit_message>
feat: update download excel, show and edit data
</commit_message>
<xml_diff>
--- a/public/assets/templates/maintenance/diesel_engine.xlsx
+++ b/public/assets/templates/maintenance/diesel_engine.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\maintenance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4BEACFFB-FC24-4D3B-88A7-13D64B323C17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79016D00-14CB-4910-A5C9-5346D163642B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{197A4A4E-22CF-4E0D-A0A6-07FA889DE95B}"/>
   </bookViews>
@@ -607,9 +607,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
@@ -640,9 +637,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
@@ -655,18 +649,24 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -676,9 +676,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -695,6 +692,9 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1139,15 +1139,15 @@
   <dimension ref="A1:M85"/>
   <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5"/>
   <cols>
-    <col min="1" max="1" width="11" style="17" customWidth="1"/>
-    <col min="2" max="2" width="3" style="17" customWidth="1"/>
-    <col min="3" max="3" width="4.26953125" style="17" customWidth="1"/>
-    <col min="4" max="4" width="23" style="17" customWidth="1"/>
-    <col min="5" max="5" width="6.26953125" style="17" customWidth="1"/>
-    <col min="6" max="6" width="2.81640625" style="17" customWidth="1"/>
-    <col min="7" max="7" width="17.81640625" style="17" customWidth="1"/>
-    <col min="8" max="8" width="4.7265625" style="17" customWidth="1"/>
-    <col min="9" max="9" width="6" style="17" customWidth="1"/>
+    <col min="1" max="1" width="11" style="15" customWidth="1"/>
+    <col min="2" max="2" width="3" style="15" customWidth="1"/>
+    <col min="3" max="3" width="4.26953125" style="15" customWidth="1"/>
+    <col min="4" max="4" width="23" style="15" customWidth="1"/>
+    <col min="5" max="5" width="6.26953125" style="15" customWidth="1"/>
+    <col min="6" max="6" width="2.81640625" style="15" customWidth="1"/>
+    <col min="7" max="7" width="17.81640625" style="15" customWidth="1"/>
+    <col min="8" max="8" width="4.7265625" style="15" customWidth="1"/>
+    <col min="9" max="9" width="6" style="15" customWidth="1"/>
     <col min="13" max="13" width="10.7265625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1185,7 +1185,7 @@
         <v>2</v>
       </c>
       <c r="C3" s="40"/>
-      <c r="D3" s="2"/>
+      <c r="D3" s="40"/>
       <c r="E3" s="41" t="s">
         <v>3</v>
       </c>
@@ -1204,7 +1204,7 @@
         <v>2</v>
       </c>
       <c r="C4" s="40"/>
-      <c r="D4" s="2"/>
+      <c r="D4" s="40"/>
       <c r="E4" s="41" t="s">
         <v>5</v>
       </c>
@@ -1215,8 +1215,8 @@
       <c r="H4" s="44"/>
       <c r="I4" s="45"/>
     </row>
-    <row r="5" spans="1:13" s="6" customFormat="1" ht="11" customHeight="1">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:13" s="5" customFormat="1" ht="11" customHeight="1">
+      <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B5" s="46" t="s">
@@ -1224,1027 +1224,1027 @@
       </c>
       <c r="C5" s="46"/>
       <c r="D5" s="46"/>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="31" t="s">
+      <c r="F5" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="G5" s="31"/>
-      <c r="H5" s="31"/>
+      <c r="G5" s="30"/>
+      <c r="H5" s="30"/>
       <c r="I5" s="47"/>
     </row>
-    <row r="6" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+    <row r="6" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A6" s="35" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="7"/>
-      <c r="C6" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="9" t="s">
+      <c r="B6" s="6"/>
+      <c r="C6" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="21"/>
-    </row>
-    <row r="7" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E6" s="16"/>
+      <c r="F6" s="18"/>
+      <c r="G6" s="18"/>
+      <c r="H6" s="18"/>
+      <c r="I6" s="19"/>
+    </row>
+    <row r="7" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A7" s="35"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="9" t="s">
+      <c r="B7" s="6"/>
+      <c r="C7" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="7"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="20"/>
-      <c r="H7" s="20"/>
-      <c r="I7" s="21"/>
-    </row>
-    <row r="8" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E7" s="16"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
+      <c r="H7" s="18"/>
+      <c r="I7" s="19"/>
+    </row>
+    <row r="8" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A8" s="35"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="9" t="s">
+      <c r="B8" s="6"/>
+      <c r="C8" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
-      <c r="H8" s="20"/>
-      <c r="I8" s="21"/>
-    </row>
-    <row r="9" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E8" s="16"/>
+      <c r="F8" s="18"/>
+      <c r="G8" s="18"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="19"/>
+    </row>
+    <row r="9" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A9" s="35"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D9" s="9" t="s">
+      <c r="B9" s="6"/>
+      <c r="C9" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="7"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
-      <c r="I9" s="21"/>
-    </row>
-    <row r="10" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E9" s="16"/>
+      <c r="F9" s="18"/>
+      <c r="G9" s="18"/>
+      <c r="H9" s="18"/>
+      <c r="I9" s="19"/>
+    </row>
+    <row r="10" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A10" s="35"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D10" s="9" t="s">
+      <c r="B10" s="6"/>
+      <c r="C10" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D10" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="E10" s="7"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
-      <c r="I10" s="21"/>
-    </row>
-    <row r="11" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E10" s="16"/>
+      <c r="F10" s="18"/>
+      <c r="G10" s="18"/>
+      <c r="H10" s="18"/>
+      <c r="I10" s="19"/>
+    </row>
+    <row r="11" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A11" s="35"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D11" s="9" t="s">
+      <c r="B11" s="6"/>
+      <c r="C11" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D11" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E11" s="7"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="21"/>
-    </row>
-    <row r="12" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E11" s="16"/>
+      <c r="F11" s="18"/>
+      <c r="G11" s="18"/>
+      <c r="H11" s="18"/>
+      <c r="I11" s="19"/>
+    </row>
+    <row r="12" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A12" s="35"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12" s="9" t="s">
+      <c r="B12" s="6"/>
+      <c r="C12" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="E12" s="7"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="20"/>
-      <c r="I12" s="21"/>
-    </row>
-    <row r="13" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E12" s="16"/>
+      <c r="F12" s="18"/>
+      <c r="G12" s="18"/>
+      <c r="H12" s="18"/>
+      <c r="I12" s="19"/>
+    </row>
+    <row r="13" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A13" s="35"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D13" s="9" t="s">
+      <c r="B13" s="6"/>
+      <c r="C13" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D13" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="E13" s="7"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="21"/>
-    </row>
-    <row r="14" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E13" s="16"/>
+      <c r="F13" s="18"/>
+      <c r="G13" s="18"/>
+      <c r="H13" s="18"/>
+      <c r="I13" s="19"/>
+    </row>
+    <row r="14" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A14" s="35"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D14" s="9" t="s">
+      <c r="B14" s="6"/>
+      <c r="C14" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D14" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="E14" s="7"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-      <c r="I14" s="21"/>
-    </row>
-    <row r="15" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E14" s="16"/>
+      <c r="F14" s="18"/>
+      <c r="G14" s="18"/>
+      <c r="H14" s="18"/>
+      <c r="I14" s="19"/>
+    </row>
+    <row r="15" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A15" s="35"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D15" s="9" t="s">
+      <c r="B15" s="6"/>
+      <c r="C15" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="E15" s="7"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="21"/>
-    </row>
-    <row r="16" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E15" s="16"/>
+      <c r="F15" s="18"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="18"/>
+      <c r="I15" s="19"/>
+    </row>
+    <row r="16" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A16" s="35"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D16" s="9" t="s">
+      <c r="B16" s="6"/>
+      <c r="C16" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D16" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="E16" s="7"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-      <c r="I16" s="21"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="18"/>
+      <c r="G16" s="18"/>
+      <c r="H16" s="18"/>
+      <c r="I16" s="19"/>
       <c r="L16" s="39"/>
       <c r="M16" s="39"/>
     </row>
-    <row r="17" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+    <row r="17" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A17" s="35"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D17" s="9" t="s">
+      <c r="B17" s="6"/>
+      <c r="C17" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="E17" s="7"/>
-      <c r="F17" s="20"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="20"/>
-      <c r="I17" s="21"/>
+      <c r="E17" s="16"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="19"/>
       <c r="L17" s="38"/>
       <c r="M17" s="38"/>
     </row>
-    <row r="18" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+    <row r="18" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A18" s="35"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D18" s="9" t="s">
+      <c r="B18" s="6"/>
+      <c r="C18" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D18" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="E18" s="7"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="20"/>
-      <c r="H18" s="20"/>
-      <c r="I18" s="21"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11"/>
-    </row>
-    <row r="19" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E18" s="16"/>
+      <c r="F18" s="18"/>
+      <c r="G18" s="18"/>
+      <c r="H18" s="18"/>
+      <c r="I18" s="19"/>
+      <c r="L18" s="10"/>
+      <c r="M18" s="10"/>
+    </row>
+    <row r="19" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A19" s="35"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="9" t="s">
+      <c r="B19" s="6"/>
+      <c r="C19" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="7"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="21"/>
-      <c r="L19" s="11"/>
-      <c r="M19" s="11"/>
-    </row>
-    <row r="20" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E19" s="16"/>
+      <c r="F19" s="18"/>
+      <c r="G19" s="18"/>
+      <c r="H19" s="18"/>
+      <c r="I19" s="19"/>
+      <c r="L19" s="10"/>
+      <c r="M19" s="10"/>
+    </row>
+    <row r="20" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A20" s="35"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D20" s="9" t="s">
+      <c r="B20" s="6"/>
+      <c r="C20" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E20" s="7"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20"/>
-      <c r="I20" s="21"/>
-      <c r="L20" s="11"/>
-      <c r="M20" s="11"/>
-    </row>
-    <row r="21" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E20" s="16"/>
+      <c r="F20" s="18"/>
+      <c r="G20" s="18"/>
+      <c r="H20" s="18"/>
+      <c r="I20" s="19"/>
+      <c r="L20" s="10"/>
+      <c r="M20" s="10"/>
+    </row>
+    <row r="21" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A21" s="35"/>
-      <c r="B21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="20"/>
-      <c r="H21" s="20"/>
-      <c r="I21" s="21"/>
+      <c r="B21" s="6"/>
+      <c r="E21" s="16"/>
+      <c r="F21" s="18"/>
+      <c r="G21" s="18"/>
+      <c r="H21" s="18"/>
+      <c r="I21" s="19"/>
       <c r="L21" s="38"/>
       <c r="M21" s="38"/>
     </row>
-    <row r="22" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+    <row r="22" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A22" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="B22" s="7"/>
-      <c r="C22" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D22" s="9" t="s">
+      <c r="B22" s="6"/>
+      <c r="C22" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="E22" s="7"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="20"/>
-      <c r="H22" s="20"/>
-      <c r="I22" s="21"/>
-    </row>
-    <row r="23" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E22" s="16"/>
+      <c r="F22" s="18"/>
+      <c r="G22" s="18"/>
+      <c r="H22" s="18"/>
+      <c r="I22" s="19"/>
+    </row>
+    <row r="23" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A23" s="35"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D23" s="9" t="s">
+      <c r="B23" s="6"/>
+      <c r="C23" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="E23" s="7"/>
-      <c r="F23" s="20"/>
-      <c r="G23" s="20"/>
-      <c r="H23" s="20"/>
-      <c r="I23" s="21"/>
-    </row>
-    <row r="24" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E23" s="16"/>
+      <c r="F23" s="18"/>
+      <c r="G23" s="18"/>
+      <c r="H23" s="18"/>
+      <c r="I23" s="19"/>
+    </row>
+    <row r="24" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A24" s="35"/>
-      <c r="B24" s="7"/>
-      <c r="C24" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D24" s="9" t="s">
+      <c r="B24" s="6"/>
+      <c r="C24" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="E24" s="7"/>
-      <c r="F24" s="20"/>
-      <c r="G24" s="20"/>
-      <c r="H24" s="20"/>
-      <c r="I24" s="21"/>
-    </row>
-    <row r="25" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E24" s="16"/>
+      <c r="F24" s="18"/>
+      <c r="G24" s="18"/>
+      <c r="H24" s="18"/>
+      <c r="I24" s="19"/>
+    </row>
+    <row r="25" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A25" s="35"/>
-      <c r="B25" s="7"/>
-      <c r="C25" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D25" s="9" t="s">
+      <c r="B25" s="6"/>
+      <c r="C25" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="E25" s="7"/>
-      <c r="F25" s="20"/>
-      <c r="G25" s="20"/>
-      <c r="H25" s="20"/>
-      <c r="I25" s="21"/>
+      <c r="E25" s="16"/>
+      <c r="F25" s="18"/>
+      <c r="G25" s="18"/>
+      <c r="H25" s="18"/>
+      <c r="I25" s="19"/>
       <c r="L25" s="36"/>
       <c r="M25" s="36"/>
     </row>
-    <row r="26" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+    <row r="26" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A26" s="35"/>
-      <c r="B26" s="7"/>
-      <c r="C26" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D26" s="9" t="s">
+      <c r="B26" s="6"/>
+      <c r="C26" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="E26" s="7"/>
-      <c r="F26" s="20"/>
-      <c r="G26" s="20"/>
-      <c r="H26" s="20"/>
-      <c r="I26" s="21"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="18"/>
+      <c r="G26" s="18"/>
+      <c r="H26" s="18"/>
+      <c r="I26" s="19"/>
       <c r="L26" s="36"/>
       <c r="M26" s="36"/>
     </row>
-    <row r="27" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+    <row r="27" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A27" s="35"/>
-      <c r="B27" s="7"/>
-      <c r="C27" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D27" s="9" t="s">
+      <c r="B27" s="6"/>
+      <c r="C27" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="E27" s="7"/>
-      <c r="F27" s="20"/>
-      <c r="G27" s="20"/>
-      <c r="H27" s="20"/>
-      <c r="I27" s="21"/>
-      <c r="L27" s="12"/>
-      <c r="M27" s="12"/>
-    </row>
-    <row r="28" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E27" s="16"/>
+      <c r="F27" s="18"/>
+      <c r="G27" s="18"/>
+      <c r="H27" s="18"/>
+      <c r="I27" s="19"/>
+      <c r="L27" s="11"/>
+      <c r="M27" s="11"/>
+    </row>
+    <row r="28" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A28" s="35"/>
-      <c r="B28" s="7"/>
-      <c r="C28" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D28" s="9" t="s">
+      <c r="B28" s="6"/>
+      <c r="C28" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D28" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="E28" s="7"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="20"/>
-      <c r="H28" s="20"/>
-      <c r="I28" s="21"/>
-      <c r="L28" s="12"/>
-      <c r="M28" s="12"/>
-    </row>
-    <row r="29" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E28" s="16"/>
+      <c r="F28" s="18"/>
+      <c r="G28" s="18"/>
+      <c r="H28" s="18"/>
+      <c r="I28" s="19"/>
+      <c r="L28" s="11"/>
+      <c r="M28" s="11"/>
+    </row>
+    <row r="29" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A29" s="35"/>
-      <c r="B29" s="7"/>
-      <c r="E29" s="7"/>
-      <c r="F29" s="20"/>
-      <c r="G29" s="20"/>
-      <c r="H29" s="20"/>
-      <c r="I29" s="21"/>
-    </row>
-    <row r="30" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="B29" s="6"/>
+      <c r="E29" s="16"/>
+      <c r="F29" s="18"/>
+      <c r="G29" s="18"/>
+      <c r="H29" s="18"/>
+      <c r="I29" s="19"/>
+    </row>
+    <row r="30" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A30" s="37" t="s">
         <v>36</v>
       </c>
-      <c r="B30" s="7"/>
-      <c r="C30" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D30" s="9" t="s">
+      <c r="B30" s="6"/>
+      <c r="C30" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D30" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="E30" s="7"/>
-      <c r="F30" s="20"/>
-      <c r="G30" s="20"/>
-      <c r="H30" s="20"/>
-      <c r="I30" s="21"/>
-    </row>
-    <row r="31" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E30" s="16"/>
+      <c r="F30" s="18"/>
+      <c r="G30" s="18"/>
+      <c r="H30" s="18"/>
+      <c r="I30" s="19"/>
+    </row>
+    <row r="31" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A31" s="37"/>
-      <c r="B31" s="7"/>
-      <c r="C31" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D31" s="9" t="s">
+      <c r="B31" s="6"/>
+      <c r="C31" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D31" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="E31" s="7"/>
-      <c r="F31" s="20"/>
-      <c r="G31" s="20"/>
-      <c r="H31" s="20"/>
-      <c r="I31" s="21"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="18"/>
+      <c r="G31" s="18"/>
+      <c r="H31" s="18"/>
+      <c r="I31" s="19"/>
       <c r="L31" s="36"/>
       <c r="M31" s="36"/>
     </row>
-    <row r="32" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+    <row r="32" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A32" s="37"/>
-      <c r="B32" s="7"/>
-      <c r="C32" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D32" s="9" t="s">
+      <c r="B32" s="6"/>
+      <c r="C32" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D32" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="E32" s="7"/>
-      <c r="F32" s="20"/>
-      <c r="G32" s="20"/>
-      <c r="H32" s="20"/>
-      <c r="I32" s="21"/>
-      <c r="L32" s="12"/>
-      <c r="M32" s="12"/>
-    </row>
-    <row r="33" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E32" s="16"/>
+      <c r="F32" s="18"/>
+      <c r="G32" s="18"/>
+      <c r="H32" s="18"/>
+      <c r="I32" s="19"/>
+      <c r="L32" s="11"/>
+      <c r="M32" s="11"/>
+    </row>
+    <row r="33" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A33" s="37"/>
-      <c r="B33" s="7"/>
-      <c r="C33" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D33" s="9" t="s">
+      <c r="B33" s="6"/>
+      <c r="C33" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="E33" s="7"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="20"/>
-      <c r="H33" s="20"/>
-      <c r="I33" s="21"/>
-      <c r="L33" s="12"/>
-      <c r="M33" s="12"/>
-    </row>
-    <row r="34" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E33" s="16"/>
+      <c r="F33" s="18"/>
+      <c r="G33" s="18"/>
+      <c r="H33" s="18"/>
+      <c r="I33" s="19"/>
+      <c r="L33" s="11"/>
+      <c r="M33" s="11"/>
+    </row>
+    <row r="34" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A34" s="37"/>
-      <c r="B34" s="7"/>
-      <c r="C34" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D34" s="9" t="s">
+      <c r="B34" s="6"/>
+      <c r="C34" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D34" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="E34" s="7"/>
-      <c r="F34" s="20"/>
-      <c r="G34" s="20"/>
-      <c r="H34" s="20"/>
-      <c r="I34" s="21"/>
-    </row>
-    <row r="35" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E34" s="16"/>
+      <c r="F34" s="18"/>
+      <c r="G34" s="18"/>
+      <c r="H34" s="18"/>
+      <c r="I34" s="19"/>
+    </row>
+    <row r="35" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A35" s="37"/>
-      <c r="B35" s="7"/>
-      <c r="C35" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D35" s="9" t="s">
+      <c r="B35" s="6"/>
+      <c r="C35" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="E35" s="7"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="20"/>
-      <c r="H35" s="20"/>
-      <c r="I35" s="21"/>
-    </row>
-    <row r="36" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E35" s="16"/>
+      <c r="F35" s="18"/>
+      <c r="G35" s="18"/>
+      <c r="H35" s="18"/>
+      <c r="I35" s="19"/>
+    </row>
+    <row r="36" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A36" s="37"/>
-      <c r="B36" s="7"/>
-      <c r="E36" s="7"/>
-      <c r="F36" s="20"/>
-      <c r="G36" s="20"/>
-      <c r="H36" s="20"/>
-      <c r="I36" s="21"/>
-    </row>
-    <row r="37" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="B36" s="6"/>
+      <c r="E36" s="16"/>
+      <c r="F36" s="18"/>
+      <c r="G36" s="18"/>
+      <c r="H36" s="18"/>
+      <c r="I36" s="19"/>
+    </row>
+    <row r="37" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A37" s="35" t="s">
         <v>43</v>
       </c>
-      <c r="B37" s="7"/>
-      <c r="C37" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D37" s="9" t="s">
+      <c r="B37" s="6"/>
+      <c r="C37" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D37" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="E37" s="7"/>
-      <c r="F37" s="20"/>
-      <c r="G37" s="20"/>
-      <c r="H37" s="20"/>
-      <c r="I37" s="21"/>
-    </row>
-    <row r="38" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E37" s="16"/>
+      <c r="F37" s="18"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="18"/>
+      <c r="I37" s="19"/>
+    </row>
+    <row r="38" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A38" s="35"/>
-      <c r="B38" s="7"/>
-      <c r="C38" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D38" s="9" t="s">
+      <c r="B38" s="6"/>
+      <c r="C38" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D38" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="E38" s="7"/>
-      <c r="F38" s="20"/>
-      <c r="G38" s="20"/>
-      <c r="H38" s="20"/>
-      <c r="I38" s="21"/>
-    </row>
-    <row r="39" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E38" s="16"/>
+      <c r="F38" s="18"/>
+      <c r="G38" s="18"/>
+      <c r="H38" s="18"/>
+      <c r="I38" s="19"/>
+    </row>
+    <row r="39" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A39" s="35"/>
-      <c r="B39" s="7"/>
-      <c r="C39" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D39" s="9" t="s">
+      <c r="B39" s="6"/>
+      <c r="C39" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D39" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="E39" s="7"/>
-      <c r="F39" s="20"/>
-      <c r="G39" s="20"/>
-      <c r="H39" s="20"/>
-      <c r="I39" s="21"/>
-    </row>
-    <row r="40" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E39" s="16"/>
+      <c r="F39" s="18"/>
+      <c r="G39" s="18"/>
+      <c r="H39" s="18"/>
+      <c r="I39" s="19"/>
+    </row>
+    <row r="40" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A40" s="35"/>
-      <c r="B40" s="7"/>
-      <c r="C40" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D40" s="9" t="s">
+      <c r="B40" s="6"/>
+      <c r="C40" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D40" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="E40" s="7"/>
-      <c r="F40" s="20"/>
-      <c r="G40" s="20"/>
-      <c r="H40" s="20"/>
-      <c r="I40" s="21"/>
-    </row>
-    <row r="41" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E40" s="16"/>
+      <c r="F40" s="18"/>
+      <c r="G40" s="18"/>
+      <c r="H40" s="18"/>
+      <c r="I40" s="19"/>
+    </row>
+    <row r="41" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A41" s="35"/>
-      <c r="B41" s="7"/>
-      <c r="C41" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D41" s="9" t="s">
+      <c r="B41" s="6"/>
+      <c r="C41" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D41" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="E41" s="7"/>
-      <c r="F41" s="20"/>
-      <c r="G41" s="20"/>
-      <c r="H41" s="20"/>
-      <c r="I41" s="21"/>
-    </row>
-    <row r="42" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E41" s="16"/>
+      <c r="F41" s="18"/>
+      <c r="G41" s="18"/>
+      <c r="H41" s="18"/>
+      <c r="I41" s="19"/>
+    </row>
+    <row r="42" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A42" s="35"/>
-      <c r="B42" s="7"/>
-      <c r="C42" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D42" s="9" t="s">
+      <c r="B42" s="6"/>
+      <c r="C42" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D42" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="E42" s="7"/>
-      <c r="F42" s="20"/>
-      <c r="G42" s="20"/>
-      <c r="H42" s="20"/>
-      <c r="I42" s="21"/>
-    </row>
-    <row r="43" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E42" s="16"/>
+      <c r="F42" s="18"/>
+      <c r="G42" s="18"/>
+      <c r="H42" s="18"/>
+      <c r="I42" s="19"/>
+    </row>
+    <row r="43" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A43" s="35"/>
-      <c r="B43" s="7"/>
-      <c r="C43" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D43" s="9" t="s">
+      <c r="B43" s="6"/>
+      <c r="C43" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D43" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="E43" s="7"/>
-      <c r="F43" s="20"/>
-      <c r="G43" s="20"/>
-      <c r="H43" s="20"/>
-      <c r="I43" s="21"/>
-    </row>
-    <row r="44" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E43" s="16"/>
+      <c r="F43" s="18"/>
+      <c r="G43" s="18"/>
+      <c r="H43" s="18"/>
+      <c r="I43" s="19"/>
+    </row>
+    <row r="44" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A44" s="35"/>
-      <c r="B44" s="7"/>
-      <c r="C44" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D44" s="9" t="s">
+      <c r="B44" s="6"/>
+      <c r="C44" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D44" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="E44" s="13"/>
-      <c r="F44" s="20"/>
-      <c r="G44" s="20"/>
-      <c r="H44" s="20"/>
-      <c r="I44" s="21"/>
-    </row>
-    <row r="45" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E44" s="17"/>
+      <c r="F44" s="18"/>
+      <c r="G44" s="18"/>
+      <c r="H44" s="18"/>
+      <c r="I44" s="19"/>
+    </row>
+    <row r="45" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A45" s="35"/>
-      <c r="B45" s="7"/>
-      <c r="C45" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D45" s="9" t="s">
+      <c r="B45" s="6"/>
+      <c r="C45" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D45" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="E45" s="13"/>
-      <c r="F45" s="20"/>
-      <c r="G45" s="20"/>
-      <c r="H45" s="20"/>
-      <c r="I45" s="21"/>
-    </row>
-    <row r="46" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E45" s="17"/>
+      <c r="F45" s="18"/>
+      <c r="G45" s="18"/>
+      <c r="H45" s="18"/>
+      <c r="I45" s="19"/>
+    </row>
+    <row r="46" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A46" s="35"/>
-      <c r="B46" s="7"/>
-      <c r="C46" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D46" s="9" t="s">
+      <c r="B46" s="6"/>
+      <c r="C46" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D46" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="E46" s="13"/>
-      <c r="F46" s="20"/>
-      <c r="G46" s="20"/>
-      <c r="H46" s="20"/>
-      <c r="I46" s="21"/>
-    </row>
-    <row r="47" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E46" s="17"/>
+      <c r="F46" s="18"/>
+      <c r="G46" s="18"/>
+      <c r="H46" s="18"/>
+      <c r="I46" s="19"/>
+    </row>
+    <row r="47" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A47" s="35"/>
-      <c r="B47" s="7"/>
-      <c r="E47" s="7"/>
-      <c r="F47" s="20"/>
-      <c r="G47" s="20"/>
-      <c r="H47" s="20"/>
-      <c r="I47" s="21"/>
-    </row>
-    <row r="48" spans="1:13" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="B47" s="6"/>
+      <c r="E47" s="16"/>
+      <c r="F47" s="18"/>
+      <c r="G47" s="18"/>
+      <c r="H47" s="18"/>
+      <c r="I47" s="19"/>
+    </row>
+    <row r="48" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A48" s="32" t="s">
         <v>54</v>
       </c>
-      <c r="B48" s="7"/>
-      <c r="C48" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D48" s="14" t="s">
+      <c r="B48" s="6"/>
+      <c r="C48" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D48" s="12" t="s">
         <v>55</v>
       </c>
-      <c r="E48" s="7"/>
-      <c r="F48" s="20"/>
-      <c r="G48" s="20"/>
-      <c r="H48" s="20"/>
-      <c r="I48" s="21"/>
-    </row>
-    <row r="49" spans="1:9" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E48" s="16"/>
+      <c r="F48" s="18"/>
+      <c r="G48" s="18"/>
+      <c r="H48" s="18"/>
+      <c r="I48" s="19"/>
+    </row>
+    <row r="49" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A49" s="33"/>
-      <c r="B49" s="7"/>
-      <c r="C49" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D49" s="14" t="s">
+      <c r="B49" s="6"/>
+      <c r="C49" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D49" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="E49" s="7"/>
-      <c r="F49" s="20"/>
-      <c r="G49" s="20"/>
-      <c r="H49" s="20"/>
-      <c r="I49" s="21"/>
-    </row>
-    <row r="50" spans="1:9" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E49" s="16"/>
+      <c r="F49" s="18"/>
+      <c r="G49" s="18"/>
+      <c r="H49" s="18"/>
+      <c r="I49" s="19"/>
+    </row>
+    <row r="50" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A50" s="33"/>
-      <c r="B50" s="7"/>
-      <c r="C50" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D50" s="14" t="s">
+      <c r="B50" s="6"/>
+      <c r="C50" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D50" s="12" t="s">
         <v>57</v>
       </c>
-      <c r="E50" s="7"/>
-      <c r="F50" s="20"/>
-      <c r="G50" s="20"/>
-      <c r="H50" s="20"/>
-      <c r="I50" s="21"/>
-    </row>
-    <row r="51" spans="1:9" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E50" s="16"/>
+      <c r="F50" s="18"/>
+      <c r="G50" s="18"/>
+      <c r="H50" s="18"/>
+      <c r="I50" s="19"/>
+    </row>
+    <row r="51" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A51" s="33"/>
-      <c r="B51" s="7"/>
-      <c r="C51" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D51" s="14" t="s">
+      <c r="B51" s="6"/>
+      <c r="C51" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D51" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="E51" s="7"/>
-      <c r="F51" s="20"/>
-      <c r="G51" s="20"/>
-      <c r="H51" s="20"/>
-      <c r="I51" s="21"/>
-    </row>
-    <row r="52" spans="1:9" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E51" s="16"/>
+      <c r="F51" s="18"/>
+      <c r="G51" s="18"/>
+      <c r="H51" s="18"/>
+      <c r="I51" s="19"/>
+    </row>
+    <row r="52" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A52" s="33"/>
-      <c r="B52" s="7"/>
-      <c r="C52" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D52" s="14" t="s">
+      <c r="B52" s="6"/>
+      <c r="C52" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D52" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="E52" s="7"/>
-      <c r="F52" s="20"/>
-      <c r="G52" s="20"/>
-      <c r="H52" s="20"/>
-      <c r="I52" s="21"/>
-    </row>
-    <row r="53" spans="1:9" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E52" s="16"/>
+      <c r="F52" s="18"/>
+      <c r="G52" s="18"/>
+      <c r="H52" s="18"/>
+      <c r="I52" s="19"/>
+    </row>
+    <row r="53" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A53" s="33"/>
-      <c r="B53" s="7"/>
-      <c r="C53" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D53" s="14" t="s">
+      <c r="B53" s="6"/>
+      <c r="C53" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D53" s="12" t="s">
         <v>60</v>
       </c>
-      <c r="E53" s="7"/>
-      <c r="F53" s="20"/>
-      <c r="G53" s="20"/>
-      <c r="H53" s="20"/>
-      <c r="I53" s="21"/>
-    </row>
-    <row r="54" spans="1:9" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E53" s="16"/>
+      <c r="F53" s="18"/>
+      <c r="G53" s="18"/>
+      <c r="H53" s="18"/>
+      <c r="I53" s="19"/>
+    </row>
+    <row r="54" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A54" s="33"/>
-      <c r="B54" s="7"/>
-      <c r="C54" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D54" s="14" t="s">
+      <c r="B54" s="6"/>
+      <c r="C54" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D54" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="E54" s="7"/>
-      <c r="F54" s="20"/>
-      <c r="G54" s="20"/>
-      <c r="H54" s="20"/>
-      <c r="I54" s="21"/>
-    </row>
-    <row r="55" spans="1:9" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E54" s="16"/>
+      <c r="F54" s="18"/>
+      <c r="G54" s="18"/>
+      <c r="H54" s="18"/>
+      <c r="I54" s="19"/>
+    </row>
+    <row r="55" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A55" s="33"/>
-      <c r="B55" s="7"/>
-      <c r="C55" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D55" s="14" t="s">
+      <c r="B55" s="6"/>
+      <c r="C55" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D55" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="E55" s="7"/>
-      <c r="F55" s="20"/>
-      <c r="G55" s="20"/>
-      <c r="H55" s="20"/>
-      <c r="I55" s="21"/>
-    </row>
-    <row r="56" spans="1:9" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E55" s="16"/>
+      <c r="F55" s="18"/>
+      <c r="G55" s="18"/>
+      <c r="H55" s="18"/>
+      <c r="I55" s="19"/>
+    </row>
+    <row r="56" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A56" s="33"/>
-      <c r="B56" s="7"/>
-      <c r="C56" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D56" s="15" t="s">
+      <c r="B56" s="6"/>
+      <c r="C56" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D56" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="E56" s="7"/>
-      <c r="F56" s="20"/>
-      <c r="G56" s="20"/>
-      <c r="H56" s="20"/>
-      <c r="I56" s="21"/>
-    </row>
-    <row r="57" spans="1:9" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E56" s="16"/>
+      <c r="F56" s="18"/>
+      <c r="G56" s="18"/>
+      <c r="H56" s="18"/>
+      <c r="I56" s="19"/>
+    </row>
+    <row r="57" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A57" s="33"/>
-      <c r="B57" s="7"/>
-      <c r="C57" s="8" t="s">
-        <v>12</v>
-      </c>
-      <c r="D57" s="15" t="s">
+      <c r="B57" s="6"/>
+      <c r="C57" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="D57" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="E57" s="7"/>
-      <c r="F57" s="20"/>
-      <c r="G57" s="20"/>
-      <c r="H57" s="20"/>
-      <c r="I57" s="21"/>
-    </row>
-    <row r="58" spans="1:9" s="10" customFormat="1" ht="9" customHeight="1">
+      <c r="E57" s="16"/>
+      <c r="F57" s="18"/>
+      <c r="G57" s="18"/>
+      <c r="H57" s="18"/>
+      <c r="I57" s="19"/>
+    </row>
+    <row r="58" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
       <c r="A58" s="34"/>
-      <c r="B58" s="7"/>
-      <c r="E58" s="7"/>
-      <c r="F58" s="20"/>
-      <c r="G58" s="20"/>
-      <c r="H58" s="20"/>
-      <c r="I58" s="21"/>
+      <c r="B58" s="6"/>
+      <c r="E58" s="16"/>
+      <c r="F58" s="18"/>
+      <c r="G58" s="18"/>
+      <c r="H58" s="18"/>
+      <c r="I58" s="19"/>
     </row>
     <row r="59" spans="1:9" ht="9" customHeight="1">
-      <c r="A59" s="26" t="s">
+      <c r="A59" s="25" t="s">
         <v>65</v>
       </c>
-      <c r="B59" s="27"/>
-      <c r="C59" s="27"/>
-      <c r="D59" s="27"/>
-      <c r="E59" s="27" t="s">
+      <c r="B59" s="26"/>
+      <c r="C59" s="26"/>
+      <c r="D59" s="26"/>
+      <c r="E59" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="F59" s="27"/>
-      <c r="G59" s="27"/>
-      <c r="H59" s="27"/>
-      <c r="I59" s="30"/>
+      <c r="F59" s="26"/>
+      <c r="G59" s="26"/>
+      <c r="H59" s="26"/>
+      <c r="I59" s="29"/>
     </row>
     <row r="60" spans="1:9" ht="9" customHeight="1">
-      <c r="A60" s="26"/>
-      <c r="B60" s="27"/>
-      <c r="C60" s="27"/>
-      <c r="D60" s="27"/>
-      <c r="E60" s="31" t="s">
+      <c r="A60" s="25"/>
+      <c r="B60" s="26"/>
+      <c r="C60" s="26"/>
+      <c r="D60" s="26"/>
+      <c r="E60" s="30" t="s">
         <v>67</v>
       </c>
-      <c r="F60" s="31"/>
-      <c r="G60" s="31"/>
-      <c r="H60" s="31"/>
-      <c r="I60" s="5" t="s">
+      <c r="F60" s="30"/>
+      <c r="G60" s="30"/>
+      <c r="H60" s="30"/>
+      <c r="I60" s="4" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="61" spans="1:9" ht="9" customHeight="1">
-      <c r="A61" s="26"/>
-      <c r="B61" s="27"/>
-      <c r="C61" s="27"/>
-      <c r="D61" s="27"/>
-      <c r="E61" s="25"/>
-      <c r="F61" s="25"/>
-      <c r="G61" s="25"/>
-      <c r="H61" s="25"/>
-      <c r="I61" s="5"/>
+      <c r="A61" s="25"/>
+      <c r="B61" s="26"/>
+      <c r="C61" s="26"/>
+      <c r="D61" s="26"/>
+      <c r="E61" s="31"/>
+      <c r="F61" s="31"/>
+      <c r="G61" s="31"/>
+      <c r="H61" s="31"/>
+      <c r="I61" s="4"/>
     </row>
     <row r="62" spans="1:9" ht="9" customHeight="1">
-      <c r="A62" s="26"/>
-      <c r="B62" s="27"/>
-      <c r="C62" s="27"/>
-      <c r="D62" s="27"/>
-      <c r="E62" s="25"/>
-      <c r="F62" s="25"/>
-      <c r="G62" s="25"/>
-      <c r="H62" s="25"/>
-      <c r="I62" s="5"/>
+      <c r="A62" s="25"/>
+      <c r="B62" s="26"/>
+      <c r="C62" s="26"/>
+      <c r="D62" s="26"/>
+      <c r="E62" s="31"/>
+      <c r="F62" s="31"/>
+      <c r="G62" s="31"/>
+      <c r="H62" s="31"/>
+      <c r="I62" s="4"/>
     </row>
     <row r="63" spans="1:9" ht="9" customHeight="1">
-      <c r="A63" s="26"/>
-      <c r="B63" s="27"/>
-      <c r="C63" s="27"/>
-      <c r="D63" s="27"/>
-      <c r="E63" s="25"/>
-      <c r="F63" s="25"/>
-      <c r="G63" s="25"/>
-      <c r="H63" s="25"/>
-      <c r="I63" s="16"/>
+      <c r="A63" s="25"/>
+      <c r="B63" s="26"/>
+      <c r="C63" s="26"/>
+      <c r="D63" s="26"/>
+      <c r="E63" s="31"/>
+      <c r="F63" s="31"/>
+      <c r="G63" s="31"/>
+      <c r="H63" s="31"/>
+      <c r="I63" s="14"/>
     </row>
     <row r="64" spans="1:9" ht="9" customHeight="1">
-      <c r="A64" s="26"/>
-      <c r="B64" s="27"/>
-      <c r="C64" s="27"/>
-      <c r="D64" s="27"/>
-      <c r="E64" s="25"/>
-      <c r="F64" s="25"/>
-      <c r="G64" s="25"/>
-      <c r="H64" s="25"/>
-      <c r="I64" s="16"/>
+      <c r="A64" s="25"/>
+      <c r="B64" s="26"/>
+      <c r="C64" s="26"/>
+      <c r="D64" s="26"/>
+      <c r="E64" s="31"/>
+      <c r="F64" s="31"/>
+      <c r="G64" s="31"/>
+      <c r="H64" s="31"/>
+      <c r="I64" s="14"/>
     </row>
     <row r="65" spans="1:9" ht="9" customHeight="1">
-      <c r="A65" s="26"/>
-      <c r="B65" s="27"/>
-      <c r="C65" s="27"/>
-      <c r="D65" s="27"/>
-      <c r="E65" s="25"/>
-      <c r="F65" s="25"/>
-      <c r="G65" s="25"/>
-      <c r="H65" s="25"/>
-      <c r="I65" s="16"/>
+      <c r="A65" s="25"/>
+      <c r="B65" s="26"/>
+      <c r="C65" s="26"/>
+      <c r="D65" s="26"/>
+      <c r="E65" s="31"/>
+      <c r="F65" s="31"/>
+      <c r="G65" s="31"/>
+      <c r="H65" s="31"/>
+      <c r="I65" s="14"/>
     </row>
     <row r="66" spans="1:9" ht="9" customHeight="1">
-      <c r="A66" s="26"/>
-      <c r="B66" s="27"/>
-      <c r="C66" s="27"/>
-      <c r="D66" s="27"/>
-      <c r="E66" s="25"/>
-      <c r="F66" s="25"/>
-      <c r="G66" s="25"/>
-      <c r="H66" s="25"/>
-      <c r="I66" s="16"/>
+      <c r="A66" s="25"/>
+      <c r="B66" s="26"/>
+      <c r="C66" s="26"/>
+      <c r="D66" s="26"/>
+      <c r="E66" s="31"/>
+      <c r="F66" s="31"/>
+      <c r="G66" s="31"/>
+      <c r="H66" s="31"/>
+      <c r="I66" s="14"/>
     </row>
     <row r="67" spans="1:9" ht="9" customHeight="1">
-      <c r="A67" s="26"/>
-      <c r="B67" s="27"/>
-      <c r="C67" s="27"/>
-      <c r="D67" s="27"/>
-      <c r="E67" s="25"/>
-      <c r="F67" s="25"/>
-      <c r="G67" s="25"/>
-      <c r="H67" s="25"/>
-      <c r="I67" s="16"/>
+      <c r="A67" s="25"/>
+      <c r="B67" s="26"/>
+      <c r="C67" s="26"/>
+      <c r="D67" s="26"/>
+      <c r="E67" s="31"/>
+      <c r="F67" s="31"/>
+      <c r="G67" s="31"/>
+      <c r="H67" s="31"/>
+      <c r="I67" s="14"/>
     </row>
     <row r="68" spans="1:9" ht="9" customHeight="1">
-      <c r="A68" s="26"/>
-      <c r="B68" s="27"/>
-      <c r="C68" s="27"/>
-      <c r="D68" s="27"/>
-      <c r="E68" s="25"/>
-      <c r="F68" s="25"/>
-      <c r="G68" s="25"/>
-      <c r="H68" s="25"/>
-      <c r="I68" s="16"/>
+      <c r="A68" s="25"/>
+      <c r="B68" s="26"/>
+      <c r="C68" s="26"/>
+      <c r="D68" s="26"/>
+      <c r="E68" s="31"/>
+      <c r="F68" s="31"/>
+      <c r="G68" s="31"/>
+      <c r="H68" s="31"/>
+      <c r="I68" s="14"/>
     </row>
     <row r="69" spans="1:9" ht="9" customHeight="1">
-      <c r="A69" s="26"/>
-      <c r="B69" s="27"/>
-      <c r="C69" s="27"/>
-      <c r="D69" s="27"/>
-      <c r="E69" s="25"/>
-      <c r="F69" s="25"/>
-      <c r="G69" s="25"/>
-      <c r="H69" s="25"/>
-      <c r="I69" s="16"/>
+      <c r="A69" s="25"/>
+      <c r="B69" s="26"/>
+      <c r="C69" s="26"/>
+      <c r="D69" s="26"/>
+      <c r="E69" s="31"/>
+      <c r="F69" s="31"/>
+      <c r="G69" s="31"/>
+      <c r="H69" s="31"/>
+      <c r="I69" s="14"/>
     </row>
     <row r="70" spans="1:9" ht="9" customHeight="1">
-      <c r="A70" s="26"/>
-      <c r="B70" s="27"/>
-      <c r="C70" s="27"/>
-      <c r="D70" s="27"/>
-      <c r="E70" s="25"/>
-      <c r="F70" s="25"/>
-      <c r="G70" s="25"/>
-      <c r="H70" s="25"/>
-      <c r="I70" s="16"/>
+      <c r="A70" s="25"/>
+      <c r="B70" s="26"/>
+      <c r="C70" s="26"/>
+      <c r="D70" s="26"/>
+      <c r="E70" s="31"/>
+      <c r="F70" s="31"/>
+      <c r="G70" s="31"/>
+      <c r="H70" s="31"/>
+      <c r="I70" s="14"/>
     </row>
     <row r="71" spans="1:9" ht="9" customHeight="1">
-      <c r="A71" s="26"/>
-      <c r="B71" s="27"/>
-      <c r="C71" s="27"/>
-      <c r="D71" s="27"/>
-      <c r="E71" s="19" t="s">
+      <c r="A71" s="25"/>
+      <c r="B71" s="26"/>
+      <c r="C71" s="26"/>
+      <c r="D71" s="26"/>
+      <c r="E71" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="F71" s="19"/>
-      <c r="G71" s="19"/>
-      <c r="H71" s="20"/>
-      <c r="I71" s="21"/>
+      <c r="F71" s="20"/>
+      <c r="G71" s="20"/>
+      <c r="H71" s="18"/>
+      <c r="I71" s="19"/>
     </row>
     <row r="72" spans="1:9" ht="9" customHeight="1">
-      <c r="A72" s="26"/>
-      <c r="B72" s="27"/>
-      <c r="C72" s="27"/>
-      <c r="D72" s="27"/>
-      <c r="E72" s="19" t="s">
+      <c r="A72" s="25"/>
+      <c r="B72" s="26"/>
+      <c r="C72" s="26"/>
+      <c r="D72" s="26"/>
+      <c r="E72" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="F72" s="19"/>
-      <c r="G72" s="19"/>
-      <c r="H72" s="20"/>
-      <c r="I72" s="21"/>
+      <c r="F72" s="20"/>
+      <c r="G72" s="20"/>
+      <c r="H72" s="18"/>
+      <c r="I72" s="19"/>
     </row>
     <row r="73" spans="1:9" ht="9" customHeight="1">
-      <c r="A73" s="26"/>
-      <c r="B73" s="27"/>
-      <c r="C73" s="27"/>
-      <c r="D73" s="27"/>
-      <c r="E73" s="19" t="s">
+      <c r="A73" s="25"/>
+      <c r="B73" s="26"/>
+      <c r="C73" s="26"/>
+      <c r="D73" s="26"/>
+      <c r="E73" s="20" t="s">
         <v>71</v>
       </c>
-      <c r="F73" s="19"/>
-      <c r="G73" s="19"/>
-      <c r="H73" s="20"/>
-      <c r="I73" s="21"/>
+      <c r="F73" s="20"/>
+      <c r="G73" s="20"/>
+      <c r="H73" s="18"/>
+      <c r="I73" s="19"/>
     </row>
     <row r="74" spans="1:9" ht="9" customHeight="1">
-      <c r="A74" s="26"/>
-      <c r="B74" s="27"/>
-      <c r="C74" s="27"/>
-      <c r="D74" s="27"/>
-      <c r="E74" s="19" t="s">
+      <c r="A74" s="25"/>
+      <c r="B74" s="26"/>
+      <c r="C74" s="26"/>
+      <c r="D74" s="26"/>
+      <c r="E74" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="F74" s="19"/>
-      <c r="G74" s="19"/>
-      <c r="H74" s="20"/>
-      <c r="I74" s="21"/>
+      <c r="F74" s="20"/>
+      <c r="G74" s="20"/>
+      <c r="H74" s="18"/>
+      <c r="I74" s="19"/>
     </row>
     <row r="75" spans="1:9" ht="9" customHeight="1">
-      <c r="A75" s="26"/>
-      <c r="B75" s="27"/>
-      <c r="C75" s="27"/>
-      <c r="D75" s="27"/>
-      <c r="E75" s="19" t="s">
+      <c r="A75" s="25"/>
+      <c r="B75" s="26"/>
+      <c r="C75" s="26"/>
+      <c r="D75" s="26"/>
+      <c r="E75" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="F75" s="19"/>
-      <c r="G75" s="19"/>
-      <c r="H75" s="20"/>
-      <c r="I75" s="21"/>
+      <c r="F75" s="20"/>
+      <c r="G75" s="20"/>
+      <c r="H75" s="18"/>
+      <c r="I75" s="19"/>
     </row>
     <row r="76" spans="1:9" ht="9" customHeight="1" thickBot="1">
-      <c r="A76" s="28"/>
-      <c r="B76" s="29"/>
-      <c r="C76" s="29"/>
-      <c r="D76" s="29"/>
+      <c r="A76" s="27"/>
+      <c r="B76" s="28"/>
+      <c r="C76" s="28"/>
+      <c r="D76" s="28"/>
       <c r="E76" s="24" t="s">
         <v>74</v>
       </c>
@@ -2254,11 +2254,11 @@
       <c r="I76" s="23"/>
     </row>
     <row r="77" spans="1:9" ht="9" customHeight="1" thickTop="1">
-      <c r="G77" s="18" t="s">
+      <c r="G77" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="H77" s="18"/>
-      <c r="I77" s="18"/>
+      <c r="H77" s="21"/>
+      <c r="I77" s="21"/>
     </row>
     <row r="78" spans="1:9" ht="9" customHeight="1">
       <c r="A78"/>
@@ -2303,27 +2303,27 @@
     <mergeCell ref="A1:C2"/>
     <mergeCell ref="D1:I1"/>
     <mergeCell ref="D2:I2"/>
-    <mergeCell ref="B3:C3"/>
     <mergeCell ref="E3:F3"/>
     <mergeCell ref="G3:I3"/>
-    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B3:D3"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="F16:I16"/>
     <mergeCell ref="E4:F4"/>
     <mergeCell ref="G4:I4"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="F5:I5"/>
-    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="B4:D4"/>
     <mergeCell ref="F10:I10"/>
     <mergeCell ref="F11:I11"/>
     <mergeCell ref="F12:I12"/>
     <mergeCell ref="F13:I13"/>
     <mergeCell ref="F14:I14"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="F16:I16"/>
     <mergeCell ref="L16:M16"/>
     <mergeCell ref="F17:I17"/>
     <mergeCell ref="L17:M17"/>
     <mergeCell ref="F18:I18"/>
     <mergeCell ref="F20:I20"/>
+    <mergeCell ref="F19:I19"/>
     <mergeCell ref="F21:I21"/>
     <mergeCell ref="L21:M21"/>
     <mergeCell ref="A22:A29"/>
@@ -2345,12 +2345,12 @@
     <mergeCell ref="A30:A36"/>
     <mergeCell ref="F30:I30"/>
     <mergeCell ref="F31:I31"/>
+    <mergeCell ref="F36:I36"/>
     <mergeCell ref="L31:M31"/>
     <mergeCell ref="F32:I32"/>
     <mergeCell ref="F33:I33"/>
     <mergeCell ref="F34:I34"/>
     <mergeCell ref="F35:I35"/>
-    <mergeCell ref="F36:I36"/>
     <mergeCell ref="A37:A47"/>
     <mergeCell ref="F37:I37"/>
     <mergeCell ref="F38:I38"/>

</xml_diff>

<commit_message>
feat: add mid column in template excel
</commit_message>
<xml_diff>
--- a/public/assets/templates/maintenance/diesel_engine.xlsx
+++ b/public/assets/templates/maintenance/diesel_engine.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\maintenance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B2BB5619-75A6-4806-ADA7-205E212DED60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B4B826-254D-475D-9091-72851F6DC0AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{197A4A4E-22CF-4E0D-A0A6-07FA889DE95B}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="83">
   <si>
     <t>LAPORAN MAINTENANCE DIESEL ENGINE</t>
   </si>
@@ -274,6 +274,9 @@
   </si>
   <si>
     <t>Lokasi</t>
+  </si>
+  <si>
+    <t>MID</t>
   </si>
 </sst>
 </file>
@@ -628,7 +631,7 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -686,12 +689,117 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -707,113 +815,17 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1198,49 +1210,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" thickTop="1">
-      <c r="A1" s="50"/>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="54" t="s">
+      <c r="A1" s="23"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="54"/>
-      <c r="F1" s="54"/>
-      <c r="G1" s="54"/>
-      <c r="H1" s="54"/>
-      <c r="I1" s="55"/>
+      <c r="E1" s="27"/>
+      <c r="F1" s="27"/>
+      <c r="G1" s="27"/>
+      <c r="H1" s="27"/>
+      <c r="I1" s="28"/>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="52"/>
-      <c r="B2" s="53"/>
-      <c r="C2" s="53"/>
-      <c r="D2" s="56" t="s">
+      <c r="A2" s="25"/>
+      <c r="B2" s="26"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="56"/>
-      <c r="F2" s="56"/>
-      <c r="G2" s="56"/>
-      <c r="H2" s="56"/>
-      <c r="I2" s="57"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+      <c r="I2" s="30"/>
     </row>
     <row r="3" spans="1:9" ht="10" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B3" s="61" t="s">
+      <c r="B3" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="49"/>
-      <c r="D3" s="49"/>
-      <c r="E3" s="42" t="s">
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="43"/>
-      <c r="G3" s="44" t="s">
+      <c r="F3" s="32"/>
+      <c r="G3" s="33" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="45"/>
-      <c r="I3" s="46"/>
+      <c r="H3" s="34"/>
+      <c r="I3" s="35"/>
     </row>
     <row r="4" spans="1:9" ht="10" customHeight="1">
       <c r="A4" s="1" t="s">
@@ -1249,17 +1261,17 @@
       <c r="B4" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="49"/>
-      <c r="D4" s="49"/>
-      <c r="E4" s="49" t="s">
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20" t="s">
         <v>80</v>
       </c>
-      <c r="F4" s="49"/>
-      <c r="G4" s="58" t="s">
+      <c r="F4" s="20"/>
+      <c r="G4" s="21" t="s">
         <v>79</v>
       </c>
-      <c r="H4" s="58"/>
-      <c r="I4" s="59"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="22"/>
     </row>
     <row r="5" spans="1:9" ht="10" customHeight="1">
       <c r="A5" s="1" t="s">
@@ -1268,17 +1280,17 @@
       <c r="B5" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="49"/>
-      <c r="D5" s="49"/>
-      <c r="E5" s="49" t="s">
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="F5" s="49"/>
-      <c r="G5" s="58" t="s">
+      <c r="F5" s="20"/>
+      <c r="G5" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="H5" s="58"/>
-      <c r="I5" s="59"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="22"/>
     </row>
     <row r="6" spans="1:9" ht="10" customHeight="1">
       <c r="A6" s="1" t="s">
@@ -1287,54 +1299,54 @@
       <c r="B6" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="49"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="42" t="s">
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="31" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="43"/>
-      <c r="G6" s="58" t="s">
+      <c r="F6" s="32"/>
+      <c r="G6" s="21" t="s">
         <v>2</v>
       </c>
-      <c r="H6" s="58"/>
-      <c r="I6" s="59"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="22"/>
     </row>
     <row r="7" spans="1:9" ht="10" customHeight="1">
       <c r="A7" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B7" s="61" t="s">
+      <c r="B7" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="49"/>
-      <c r="D7" s="49"/>
-      <c r="E7" s="60"/>
-      <c r="F7" s="60"/>
-      <c r="G7" s="44"/>
-      <c r="H7" s="45"/>
-      <c r="I7" s="46"/>
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
+      <c r="G7" s="33"/>
+      <c r="H7" s="34"/>
+      <c r="I7" s="35"/>
     </row>
     <row r="8" spans="1:9" s="5" customFormat="1" ht="11" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="47" t="s">
+      <c r="B8" s="38" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="47"/>
-      <c r="D8" s="47"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
       <c r="E8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F8" s="32" t="s">
+      <c r="F8" s="39" t="s">
         <v>8</v>
       </c>
-      <c r="G8" s="32"/>
-      <c r="H8" s="32"/>
-      <c r="I8" s="48"/>
+      <c r="G8" s="39"/>
+      <c r="H8" s="39"/>
+      <c r="I8" s="40"/>
     </row>
     <row r="9" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A9" s="37" t="s">
+      <c r="A9" s="44" t="s">
         <v>9</v>
       </c>
       <c r="B9" s="6"/>
@@ -1345,13 +1357,13 @@
         <v>11</v>
       </c>
       <c r="E9" s="16"/>
-      <c r="F9" s="19"/>
-      <c r="G9" s="19"/>
-      <c r="H9" s="19"/>
-      <c r="I9" s="20"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="36"/>
+      <c r="H9" s="36"/>
+      <c r="I9" s="37"/>
     </row>
     <row r="10" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A10" s="37"/>
+      <c r="A10" s="44"/>
       <c r="B10" s="6"/>
       <c r="C10" s="7" t="s">
         <v>10</v>
@@ -1360,13 +1372,13 @@
         <v>12</v>
       </c>
       <c r="E10" s="16"/>
-      <c r="F10" s="19"/>
-      <c r="G10" s="19"/>
-      <c r="H10" s="19"/>
-      <c r="I10" s="20"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="36"/>
+      <c r="H10" s="36"/>
+      <c r="I10" s="37"/>
     </row>
     <row r="11" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A11" s="37"/>
+      <c r="A11" s="44"/>
       <c r="B11" s="6"/>
       <c r="C11" s="7" t="s">
         <v>10</v>
@@ -1375,13 +1387,13 @@
         <v>13</v>
       </c>
       <c r="E11" s="16"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="20"/>
+      <c r="F11" s="36"/>
+      <c r="G11" s="36"/>
+      <c r="H11" s="36"/>
+      <c r="I11" s="37"/>
     </row>
     <row r="12" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A12" s="37"/>
+      <c r="A12" s="44"/>
       <c r="B12" s="6"/>
       <c r="C12" s="7" t="s">
         <v>10</v>
@@ -1390,13 +1402,13 @@
         <v>14</v>
       </c>
       <c r="E12" s="16"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="19"/>
-      <c r="H12" s="19"/>
-      <c r="I12" s="20"/>
+      <c r="F12" s="36"/>
+      <c r="G12" s="36"/>
+      <c r="H12" s="36"/>
+      <c r="I12" s="37"/>
     </row>
     <row r="13" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A13" s="37"/>
+      <c r="A13" s="44"/>
       <c r="B13" s="6"/>
       <c r="C13" s="7" t="s">
         <v>10</v>
@@ -1405,13 +1417,13 @@
         <v>15</v>
       </c>
       <c r="E13" s="16"/>
-      <c r="F13" s="19"/>
-      <c r="G13" s="19"/>
-      <c r="H13" s="19"/>
-      <c r="I13" s="20"/>
+      <c r="F13" s="36"/>
+      <c r="G13" s="36"/>
+      <c r="H13" s="36"/>
+      <c r="I13" s="37"/>
     </row>
     <row r="14" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A14" s="37"/>
+      <c r="A14" s="44"/>
       <c r="B14" s="6"/>
       <c r="C14" s="7" t="s">
         <v>10</v>
@@ -1420,13 +1432,13 @@
         <v>16</v>
       </c>
       <c r="E14" s="16"/>
-      <c r="F14" s="19"/>
-      <c r="G14" s="19"/>
-      <c r="H14" s="19"/>
-      <c r="I14" s="20"/>
+      <c r="F14" s="36"/>
+      <c r="G14" s="36"/>
+      <c r="H14" s="36"/>
+      <c r="I14" s="37"/>
     </row>
     <row r="15" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A15" s="37"/>
+      <c r="A15" s="44"/>
       <c r="B15" s="6"/>
       <c r="C15" s="7" t="s">
         <v>10</v>
@@ -1435,13 +1447,13 @@
         <v>17</v>
       </c>
       <c r="E15" s="16"/>
-      <c r="F15" s="19"/>
-      <c r="G15" s="19"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="20"/>
+      <c r="F15" s="36"/>
+      <c r="G15" s="36"/>
+      <c r="H15" s="36"/>
+      <c r="I15" s="37"/>
     </row>
     <row r="16" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A16" s="37"/>
+      <c r="A16" s="44"/>
       <c r="B16" s="6"/>
       <c r="C16" s="7" t="s">
         <v>10</v>
@@ -1450,13 +1462,13 @@
         <v>18</v>
       </c>
       <c r="E16" s="16"/>
-      <c r="F16" s="19"/>
-      <c r="G16" s="19"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="20"/>
+      <c r="F16" s="36"/>
+      <c r="G16" s="36"/>
+      <c r="H16" s="36"/>
+      <c r="I16" s="37"/>
     </row>
     <row r="17" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A17" s="37"/>
+      <c r="A17" s="44"/>
       <c r="B17" s="6"/>
       <c r="C17" s="7" t="s">
         <v>10</v>
@@ -1465,13 +1477,13 @@
         <v>19</v>
       </c>
       <c r="E17" s="16"/>
-      <c r="F17" s="19"/>
-      <c r="G17" s="19"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="20"/>
+      <c r="F17" s="36"/>
+      <c r="G17" s="36"/>
+      <c r="H17" s="36"/>
+      <c r="I17" s="37"/>
     </row>
     <row r="18" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A18" s="37"/>
+      <c r="A18" s="44"/>
       <c r="B18" s="6"/>
       <c r="C18" s="7" t="s">
         <v>10</v>
@@ -1480,13 +1492,13 @@
         <v>20</v>
       </c>
       <c r="E18" s="16"/>
-      <c r="F18" s="19"/>
-      <c r="G18" s="19"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="20"/>
+      <c r="F18" s="36"/>
+      <c r="G18" s="36"/>
+      <c r="H18" s="36"/>
+      <c r="I18" s="37"/>
     </row>
     <row r="19" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A19" s="37"/>
+      <c r="A19" s="44"/>
       <c r="B19" s="6"/>
       <c r="C19" s="7" t="s">
         <v>10</v>
@@ -1495,15 +1507,15 @@
         <v>21</v>
       </c>
       <c r="E19" s="16"/>
-      <c r="F19" s="19"/>
-      <c r="G19" s="19"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="20"/>
-      <c r="L19" s="41"/>
-      <c r="M19" s="41"/>
+      <c r="F19" s="36"/>
+      <c r="G19" s="36"/>
+      <c r="H19" s="36"/>
+      <c r="I19" s="37"/>
+      <c r="L19" s="42"/>
+      <c r="M19" s="42"/>
     </row>
     <row r="20" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A20" s="37"/>
+      <c r="A20" s="44"/>
       <c r="B20" s="6"/>
       <c r="C20" s="7" t="s">
         <v>10</v>
@@ -1512,15 +1524,15 @@
         <v>22</v>
       </c>
       <c r="E20" s="16"/>
-      <c r="F20" s="19"/>
-      <c r="G20" s="19"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="20"/>
-      <c r="L20" s="40"/>
-      <c r="M20" s="40"/>
+      <c r="F20" s="36"/>
+      <c r="G20" s="36"/>
+      <c r="H20" s="36"/>
+      <c r="I20" s="37"/>
+      <c r="L20" s="43"/>
+      <c r="M20" s="43"/>
     </row>
     <row r="21" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A21" s="37"/>
+      <c r="A21" s="44"/>
       <c r="B21" s="6"/>
       <c r="C21" s="7" t="s">
         <v>10</v>
@@ -1529,15 +1541,15 @@
         <v>23</v>
       </c>
       <c r="E21" s="16"/>
-      <c r="F21" s="19"/>
-      <c r="G21" s="19"/>
-      <c r="H21" s="19"/>
-      <c r="I21" s="20"/>
+      <c r="F21" s="36"/>
+      <c r="G21" s="36"/>
+      <c r="H21" s="36"/>
+      <c r="I21" s="37"/>
       <c r="L21" s="10"/>
       <c r="M21" s="10"/>
     </row>
     <row r="22" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A22" s="37"/>
+      <c r="A22" s="44"/>
       <c r="B22" s="6"/>
       <c r="C22" s="7" t="s">
         <v>10</v>
@@ -1546,15 +1558,15 @@
         <v>24</v>
       </c>
       <c r="E22" s="16"/>
-      <c r="F22" s="19"/>
-      <c r="G22" s="19"/>
-      <c r="H22" s="19"/>
-      <c r="I22" s="20"/>
+      <c r="F22" s="36"/>
+      <c r="G22" s="36"/>
+      <c r="H22" s="36"/>
+      <c r="I22" s="37"/>
       <c r="L22" s="10"/>
       <c r="M22" s="10"/>
     </row>
     <row r="23" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A23" s="37"/>
+      <c r="A23" s="44"/>
       <c r="B23" s="6"/>
       <c r="C23" s="7" t="s">
         <v>10</v>
@@ -1563,26 +1575,26 @@
         <v>25</v>
       </c>
       <c r="E23" s="16"/>
-      <c r="F23" s="19"/>
-      <c r="G23" s="19"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="20"/>
+      <c r="F23" s="36"/>
+      <c r="G23" s="36"/>
+      <c r="H23" s="36"/>
+      <c r="I23" s="37"/>
       <c r="L23" s="10"/>
       <c r="M23" s="10"/>
     </row>
     <row r="24" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A24" s="37"/>
+      <c r="A24" s="44"/>
       <c r="B24" s="6"/>
       <c r="E24" s="16"/>
-      <c r="F24" s="19"/>
-      <c r="G24" s="19"/>
-      <c r="H24" s="19"/>
-      <c r="I24" s="20"/>
-      <c r="L24" s="40"/>
-      <c r="M24" s="40"/>
+      <c r="F24" s="36"/>
+      <c r="G24" s="36"/>
+      <c r="H24" s="36"/>
+      <c r="I24" s="37"/>
+      <c r="L24" s="43"/>
+      <c r="M24" s="43"/>
     </row>
     <row r="25" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A25" s="37" t="s">
+      <c r="A25" s="44" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="6"/>
@@ -1593,13 +1605,13 @@
         <v>27</v>
       </c>
       <c r="E25" s="16"/>
-      <c r="F25" s="19"/>
-      <c r="G25" s="19"/>
-      <c r="H25" s="19"/>
-      <c r="I25" s="20"/>
+      <c r="F25" s="36"/>
+      <c r="G25" s="36"/>
+      <c r="H25" s="36"/>
+      <c r="I25" s="37"/>
     </row>
     <row r="26" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A26" s="37"/>
+      <c r="A26" s="44"/>
       <c r="B26" s="6"/>
       <c r="C26" s="7" t="s">
         <v>10</v>
@@ -1608,13 +1620,13 @@
         <v>28</v>
       </c>
       <c r="E26" s="16"/>
-      <c r="F26" s="19"/>
-      <c r="G26" s="19"/>
-      <c r="H26" s="19"/>
-      <c r="I26" s="20"/>
+      <c r="F26" s="36"/>
+      <c r="G26" s="36"/>
+      <c r="H26" s="36"/>
+      <c r="I26" s="37"/>
     </row>
     <row r="27" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A27" s="37"/>
+      <c r="A27" s="44"/>
       <c r="B27" s="6"/>
       <c r="C27" s="7" t="s">
         <v>10</v>
@@ -1623,13 +1635,13 @@
         <v>29</v>
       </c>
       <c r="E27" s="16"/>
-      <c r="F27" s="19"/>
-      <c r="G27" s="19"/>
-      <c r="H27" s="19"/>
-      <c r="I27" s="20"/>
+      <c r="F27" s="36"/>
+      <c r="G27" s="36"/>
+      <c r="H27" s="36"/>
+      <c r="I27" s="37"/>
     </row>
     <row r="28" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A28" s="37"/>
+      <c r="A28" s="44"/>
       <c r="B28" s="6"/>
       <c r="C28" s="7" t="s">
         <v>10</v>
@@ -1638,15 +1650,15 @@
         <v>30</v>
       </c>
       <c r="E28" s="16"/>
-      <c r="F28" s="19"/>
-      <c r="G28" s="19"/>
-      <c r="H28" s="19"/>
-      <c r="I28" s="20"/>
-      <c r="L28" s="38"/>
-      <c r="M28" s="38"/>
+      <c r="F28" s="36"/>
+      <c r="G28" s="36"/>
+      <c r="H28" s="36"/>
+      <c r="I28" s="37"/>
+      <c r="L28" s="45"/>
+      <c r="M28" s="45"/>
     </row>
     <row r="29" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A29" s="37"/>
+      <c r="A29" s="44"/>
       <c r="B29" s="6"/>
       <c r="C29" s="7" t="s">
         <v>10</v>
@@ -1655,15 +1667,15 @@
         <v>31</v>
       </c>
       <c r="E29" s="16"/>
-      <c r="F29" s="19"/>
-      <c r="G29" s="19"/>
-      <c r="H29" s="19"/>
-      <c r="I29" s="20"/>
-      <c r="L29" s="38"/>
-      <c r="M29" s="38"/>
+      <c r="F29" s="36"/>
+      <c r="G29" s="36"/>
+      <c r="H29" s="36"/>
+      <c r="I29" s="37"/>
+      <c r="L29" s="45"/>
+      <c r="M29" s="45"/>
     </row>
     <row r="30" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A30" s="37"/>
+      <c r="A30" s="44"/>
       <c r="B30" s="6"/>
       <c r="C30" s="7" t="s">
         <v>10</v>
@@ -1672,15 +1684,15 @@
         <v>32</v>
       </c>
       <c r="E30" s="16"/>
-      <c r="F30" s="19"/>
-      <c r="G30" s="19"/>
-      <c r="H30" s="19"/>
-      <c r="I30" s="20"/>
+      <c r="F30" s="36"/>
+      <c r="G30" s="36"/>
+      <c r="H30" s="36"/>
+      <c r="I30" s="37"/>
       <c r="L30" s="11"/>
       <c r="M30" s="11"/>
     </row>
     <row r="31" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A31" s="37"/>
+      <c r="A31" s="44"/>
       <c r="B31" s="6"/>
       <c r="C31" s="7" t="s">
         <v>10</v>
@@ -1689,24 +1701,24 @@
         <v>33</v>
       </c>
       <c r="E31" s="16"/>
-      <c r="F31" s="19"/>
-      <c r="G31" s="19"/>
-      <c r="H31" s="19"/>
-      <c r="I31" s="20"/>
+      <c r="F31" s="36"/>
+      <c r="G31" s="36"/>
+      <c r="H31" s="36"/>
+      <c r="I31" s="37"/>
       <c r="L31" s="11"/>
       <c r="M31" s="11"/>
     </row>
     <row r="32" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A32" s="37"/>
+      <c r="A32" s="44"/>
       <c r="B32" s="6"/>
       <c r="E32" s="16"/>
-      <c r="F32" s="19"/>
-      <c r="G32" s="19"/>
-      <c r="H32" s="19"/>
-      <c r="I32" s="20"/>
+      <c r="F32" s="36"/>
+      <c r="G32" s="36"/>
+      <c r="H32" s="36"/>
+      <c r="I32" s="37"/>
     </row>
     <row r="33" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A33" s="39" t="s">
+      <c r="A33" s="46" t="s">
         <v>34</v>
       </c>
       <c r="B33" s="6"/>
@@ -1717,13 +1729,13 @@
         <v>35</v>
       </c>
       <c r="E33" s="16"/>
-      <c r="F33" s="19"/>
-      <c r="G33" s="19"/>
-      <c r="H33" s="19"/>
-      <c r="I33" s="20"/>
+      <c r="F33" s="36"/>
+      <c r="G33" s="36"/>
+      <c r="H33" s="36"/>
+      <c r="I33" s="37"/>
     </row>
     <row r="34" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A34" s="39"/>
+      <c r="A34" s="46"/>
       <c r="B34" s="6"/>
       <c r="C34" s="7" t="s">
         <v>10</v>
@@ -1732,15 +1744,15 @@
         <v>36</v>
       </c>
       <c r="E34" s="16"/>
-      <c r="F34" s="19"/>
-      <c r="G34" s="19"/>
-      <c r="H34" s="19"/>
-      <c r="I34" s="20"/>
-      <c r="L34" s="38"/>
-      <c r="M34" s="38"/>
+      <c r="F34" s="36"/>
+      <c r="G34" s="36"/>
+      <c r="H34" s="36"/>
+      <c r="I34" s="37"/>
+      <c r="L34" s="45"/>
+      <c r="M34" s="45"/>
     </row>
     <row r="35" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A35" s="39"/>
+      <c r="A35" s="46"/>
       <c r="B35" s="6"/>
       <c r="C35" s="7" t="s">
         <v>10</v>
@@ -1749,15 +1761,15 @@
         <v>37</v>
       </c>
       <c r="E35" s="16"/>
-      <c r="F35" s="19"/>
-      <c r="G35" s="19"/>
-      <c r="H35" s="19"/>
-      <c r="I35" s="20"/>
+      <c r="F35" s="36"/>
+      <c r="G35" s="36"/>
+      <c r="H35" s="36"/>
+      <c r="I35" s="37"/>
       <c r="L35" s="11"/>
       <c r="M35" s="11"/>
     </row>
     <row r="36" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A36" s="39"/>
+      <c r="A36" s="46"/>
       <c r="B36" s="6"/>
       <c r="C36" s="7" t="s">
         <v>10</v>
@@ -1766,15 +1778,15 @@
         <v>38</v>
       </c>
       <c r="E36" s="16"/>
-      <c r="F36" s="19"/>
-      <c r="G36" s="19"/>
-      <c r="H36" s="19"/>
-      <c r="I36" s="20"/>
+      <c r="F36" s="36"/>
+      <c r="G36" s="36"/>
+      <c r="H36" s="36"/>
+      <c r="I36" s="37"/>
       <c r="L36" s="11"/>
       <c r="M36" s="11"/>
     </row>
     <row r="37" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A37" s="39"/>
+      <c r="A37" s="46"/>
       <c r="B37" s="6"/>
       <c r="C37" s="7" t="s">
         <v>10</v>
@@ -1783,13 +1795,13 @@
         <v>39</v>
       </c>
       <c r="E37" s="16"/>
-      <c r="F37" s="19"/>
-      <c r="G37" s="19"/>
-      <c r="H37" s="19"/>
-      <c r="I37" s="20"/>
+      <c r="F37" s="36"/>
+      <c r="G37" s="36"/>
+      <c r="H37" s="36"/>
+      <c r="I37" s="37"/>
     </row>
     <row r="38" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A38" s="39"/>
+      <c r="A38" s="46"/>
       <c r="B38" s="6"/>
       <c r="C38" s="7" t="s">
         <v>10</v>
@@ -1798,22 +1810,22 @@
         <v>40</v>
       </c>
       <c r="E38" s="16"/>
-      <c r="F38" s="19"/>
-      <c r="G38" s="19"/>
-      <c r="H38" s="19"/>
-      <c r="I38" s="20"/>
+      <c r="F38" s="36"/>
+      <c r="G38" s="36"/>
+      <c r="H38" s="36"/>
+      <c r="I38" s="37"/>
     </row>
     <row r="39" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A39" s="39"/>
+      <c r="A39" s="46"/>
       <c r="B39" s="6"/>
       <c r="E39" s="16"/>
-      <c r="F39" s="19"/>
-      <c r="G39" s="19"/>
-      <c r="H39" s="19"/>
-      <c r="I39" s="20"/>
+      <c r="F39" s="36"/>
+      <c r="G39" s="36"/>
+      <c r="H39" s="36"/>
+      <c r="I39" s="37"/>
     </row>
     <row r="40" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A40" s="37" t="s">
+      <c r="A40" s="44" t="s">
         <v>41</v>
       </c>
       <c r="B40" s="6"/>
@@ -1824,13 +1836,13 @@
         <v>42</v>
       </c>
       <c r="E40" s="16"/>
-      <c r="F40" s="19"/>
-      <c r="G40" s="19"/>
-      <c r="H40" s="19"/>
-      <c r="I40" s="20"/>
+      <c r="F40" s="36"/>
+      <c r="G40" s="36"/>
+      <c r="H40" s="36"/>
+      <c r="I40" s="37"/>
     </row>
     <row r="41" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A41" s="37"/>
+      <c r="A41" s="44"/>
       <c r="B41" s="6"/>
       <c r="C41" s="7" t="s">
         <v>10</v>
@@ -1839,13 +1851,13 @@
         <v>43</v>
       </c>
       <c r="E41" s="16"/>
-      <c r="F41" s="19"/>
-      <c r="G41" s="19"/>
-      <c r="H41" s="19"/>
-      <c r="I41" s="20"/>
+      <c r="F41" s="36"/>
+      <c r="G41" s="36"/>
+      <c r="H41" s="36"/>
+      <c r="I41" s="37"/>
     </row>
     <row r="42" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A42" s="37"/>
+      <c r="A42" s="44"/>
       <c r="B42" s="6"/>
       <c r="C42" s="7" t="s">
         <v>10</v>
@@ -1854,13 +1866,13 @@
         <v>44</v>
       </c>
       <c r="E42" s="16"/>
-      <c r="F42" s="19"/>
-      <c r="G42" s="19"/>
-      <c r="H42" s="19"/>
-      <c r="I42" s="20"/>
+      <c r="F42" s="36"/>
+      <c r="G42" s="36"/>
+      <c r="H42" s="36"/>
+      <c r="I42" s="37"/>
     </row>
     <row r="43" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A43" s="37"/>
+      <c r="A43" s="44"/>
       <c r="B43" s="6"/>
       <c r="C43" s="7" t="s">
         <v>10</v>
@@ -1869,13 +1881,13 @@
         <v>45</v>
       </c>
       <c r="E43" s="16"/>
-      <c r="F43" s="19"/>
-      <c r="G43" s="19"/>
-      <c r="H43" s="19"/>
-      <c r="I43" s="20"/>
+      <c r="F43" s="36"/>
+      <c r="G43" s="36"/>
+      <c r="H43" s="36"/>
+      <c r="I43" s="37"/>
     </row>
     <row r="44" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A44" s="37"/>
+      <c r="A44" s="44"/>
       <c r="B44" s="6"/>
       <c r="C44" s="7" t="s">
         <v>10</v>
@@ -1884,13 +1896,13 @@
         <v>46</v>
       </c>
       <c r="E44" s="16"/>
-      <c r="F44" s="19"/>
-      <c r="G44" s="19"/>
-      <c r="H44" s="19"/>
-      <c r="I44" s="20"/>
+      <c r="F44" s="36"/>
+      <c r="G44" s="36"/>
+      <c r="H44" s="36"/>
+      <c r="I44" s="37"/>
     </row>
     <row r="45" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A45" s="37"/>
+      <c r="A45" s="44"/>
       <c r="B45" s="6"/>
       <c r="C45" s="7" t="s">
         <v>10</v>
@@ -1899,13 +1911,13 @@
         <v>47</v>
       </c>
       <c r="E45" s="16"/>
-      <c r="F45" s="19"/>
-      <c r="G45" s="19"/>
-      <c r="H45" s="19"/>
-      <c r="I45" s="20"/>
+      <c r="F45" s="36"/>
+      <c r="G45" s="36"/>
+      <c r="H45" s="36"/>
+      <c r="I45" s="37"/>
     </row>
     <row r="46" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A46" s="37"/>
+      <c r="A46" s="44"/>
       <c r="B46" s="6"/>
       <c r="C46" s="7" t="s">
         <v>10</v>
@@ -1914,13 +1926,13 @@
         <v>48</v>
       </c>
       <c r="E46" s="16"/>
-      <c r="F46" s="19"/>
-      <c r="G46" s="19"/>
-      <c r="H46" s="19"/>
-      <c r="I46" s="20"/>
+      <c r="F46" s="36"/>
+      <c r="G46" s="36"/>
+      <c r="H46" s="36"/>
+      <c r="I46" s="37"/>
     </row>
     <row r="47" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A47" s="37"/>
+      <c r="A47" s="44"/>
       <c r="B47" s="6"/>
       <c r="C47" s="7" t="s">
         <v>10</v>
@@ -1929,13 +1941,13 @@
         <v>49</v>
       </c>
       <c r="E47" s="17"/>
-      <c r="F47" s="19"/>
-      <c r="G47" s="19"/>
-      <c r="H47" s="19"/>
-      <c r="I47" s="20"/>
+      <c r="F47" s="36"/>
+      <c r="G47" s="36"/>
+      <c r="H47" s="36"/>
+      <c r="I47" s="37"/>
     </row>
     <row r="48" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A48" s="37"/>
+      <c r="A48" s="44"/>
       <c r="B48" s="6"/>
       <c r="C48" s="7" t="s">
         <v>10</v>
@@ -1944,13 +1956,13 @@
         <v>50</v>
       </c>
       <c r="E48" s="17"/>
-      <c r="F48" s="19"/>
-      <c r="G48" s="19"/>
-      <c r="H48" s="19"/>
-      <c r="I48" s="20"/>
+      <c r="F48" s="36"/>
+      <c r="G48" s="36"/>
+      <c r="H48" s="36"/>
+      <c r="I48" s="37"/>
     </row>
     <row r="49" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A49" s="37"/>
+      <c r="A49" s="44"/>
       <c r="B49" s="6"/>
       <c r="C49" s="7" t="s">
         <v>10</v>
@@ -1959,22 +1971,22 @@
         <v>51</v>
       </c>
       <c r="E49" s="17"/>
-      <c r="F49" s="19"/>
-      <c r="G49" s="19"/>
-      <c r="H49" s="19"/>
-      <c r="I49" s="20"/>
+      <c r="F49" s="36"/>
+      <c r="G49" s="36"/>
+      <c r="H49" s="36"/>
+      <c r="I49" s="37"/>
     </row>
     <row r="50" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A50" s="37"/>
+      <c r="A50" s="44"/>
       <c r="B50" s="6"/>
       <c r="E50" s="16"/>
-      <c r="F50" s="19"/>
-      <c r="G50" s="19"/>
-      <c r="H50" s="19"/>
-      <c r="I50" s="20"/>
+      <c r="F50" s="36"/>
+      <c r="G50" s="36"/>
+      <c r="H50" s="36"/>
+      <c r="I50" s="37"/>
     </row>
     <row r="51" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A51" s="34" t="s">
+      <c r="A51" s="53" t="s">
         <v>52</v>
       </c>
       <c r="B51" s="6"/>
@@ -1985,13 +1997,13 @@
         <v>53</v>
       </c>
       <c r="E51" s="16"/>
-      <c r="F51" s="19"/>
-      <c r="G51" s="19"/>
-      <c r="H51" s="19"/>
-      <c r="I51" s="20"/>
+      <c r="F51" s="36"/>
+      <c r="G51" s="36"/>
+      <c r="H51" s="36"/>
+      <c r="I51" s="37"/>
     </row>
     <row r="52" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A52" s="35"/>
+      <c r="A52" s="54"/>
       <c r="B52" s="6"/>
       <c r="C52" s="7" t="s">
         <v>10</v>
@@ -2000,13 +2012,13 @@
         <v>54</v>
       </c>
       <c r="E52" s="16"/>
-      <c r="F52" s="19"/>
-      <c r="G52" s="19"/>
-      <c r="H52" s="19"/>
-      <c r="I52" s="20"/>
+      <c r="F52" s="36"/>
+      <c r="G52" s="36"/>
+      <c r="H52" s="36"/>
+      <c r="I52" s="37"/>
     </row>
     <row r="53" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A53" s="35"/>
+      <c r="A53" s="54"/>
       <c r="B53" s="6"/>
       <c r="C53" s="7" t="s">
         <v>10</v>
@@ -2015,13 +2027,13 @@
         <v>55</v>
       </c>
       <c r="E53" s="16"/>
-      <c r="F53" s="19"/>
-      <c r="G53" s="19"/>
-      <c r="H53" s="19"/>
-      <c r="I53" s="20"/>
+      <c r="F53" s="36"/>
+      <c r="G53" s="36"/>
+      <c r="H53" s="36"/>
+      <c r="I53" s="37"/>
     </row>
     <row r="54" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A54" s="35"/>
+      <c r="A54" s="54"/>
       <c r="B54" s="6"/>
       <c r="C54" s="7" t="s">
         <v>10</v>
@@ -2030,13 +2042,13 @@
         <v>56</v>
       </c>
       <c r="E54" s="16"/>
-      <c r="F54" s="19"/>
-      <c r="G54" s="19"/>
-      <c r="H54" s="19"/>
-      <c r="I54" s="20"/>
+      <c r="F54" s="36"/>
+      <c r="G54" s="36"/>
+      <c r="H54" s="36"/>
+      <c r="I54" s="37"/>
     </row>
     <row r="55" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A55" s="35"/>
+      <c r="A55" s="54"/>
       <c r="B55" s="6"/>
       <c r="C55" s="7" t="s">
         <v>10</v>
@@ -2045,13 +2057,13 @@
         <v>57</v>
       </c>
       <c r="E55" s="16"/>
-      <c r="F55" s="19"/>
-      <c r="G55" s="19"/>
-      <c r="H55" s="19"/>
-      <c r="I55" s="20"/>
+      <c r="F55" s="36"/>
+      <c r="G55" s="36"/>
+      <c r="H55" s="36"/>
+      <c r="I55" s="37"/>
     </row>
     <row r="56" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A56" s="35"/>
+      <c r="A56" s="54"/>
       <c r="B56" s="6"/>
       <c r="C56" s="7" t="s">
         <v>10</v>
@@ -2060,13 +2072,13 @@
         <v>58</v>
       </c>
       <c r="E56" s="16"/>
-      <c r="F56" s="19"/>
-      <c r="G56" s="19"/>
-      <c r="H56" s="19"/>
-      <c r="I56" s="20"/>
+      <c r="F56" s="36"/>
+      <c r="G56" s="36"/>
+      <c r="H56" s="36"/>
+      <c r="I56" s="37"/>
     </row>
     <row r="57" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A57" s="35"/>
+      <c r="A57" s="54"/>
       <c r="B57" s="6"/>
       <c r="C57" s="7" t="s">
         <v>10</v>
@@ -2075,13 +2087,13 @@
         <v>59</v>
       </c>
       <c r="E57" s="16"/>
-      <c r="F57" s="19"/>
-      <c r="G57" s="19"/>
-      <c r="H57" s="19"/>
-      <c r="I57" s="20"/>
+      <c r="F57" s="36"/>
+      <c r="G57" s="36"/>
+      <c r="H57" s="36"/>
+      <c r="I57" s="37"/>
     </row>
     <row r="58" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A58" s="35"/>
+      <c r="A58" s="54"/>
       <c r="B58" s="6"/>
       <c r="C58" s="7" t="s">
         <v>10</v>
@@ -2090,13 +2102,13 @@
         <v>60</v>
       </c>
       <c r="E58" s="16"/>
-      <c r="F58" s="19"/>
-      <c r="G58" s="19"/>
-      <c r="H58" s="19"/>
-      <c r="I58" s="20"/>
+      <c r="F58" s="36"/>
+      <c r="G58" s="36"/>
+      <c r="H58" s="36"/>
+      <c r="I58" s="37"/>
     </row>
     <row r="59" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A59" s="35"/>
+      <c r="A59" s="54"/>
       <c r="B59" s="6"/>
       <c r="C59" s="7" t="s">
         <v>10</v>
@@ -2105,13 +2117,13 @@
         <v>61</v>
       </c>
       <c r="E59" s="16"/>
-      <c r="F59" s="19"/>
-      <c r="G59" s="19"/>
-      <c r="H59" s="19"/>
-      <c r="I59" s="20"/>
+      <c r="F59" s="36"/>
+      <c r="G59" s="36"/>
+      <c r="H59" s="36"/>
+      <c r="I59" s="37"/>
     </row>
     <row r="60" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A60" s="35"/>
+      <c r="A60" s="54"/>
       <c r="B60" s="6"/>
       <c r="C60" s="7" t="s">
         <v>10</v>
@@ -2120,244 +2132,246 @@
         <v>62</v>
       </c>
       <c r="E60" s="16"/>
-      <c r="F60" s="19"/>
-      <c r="G60" s="19"/>
-      <c r="H60" s="19"/>
-      <c r="I60" s="20"/>
+      <c r="F60" s="36"/>
+      <c r="G60" s="36"/>
+      <c r="H60" s="36"/>
+      <c r="I60" s="37"/>
     </row>
     <row r="61" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A61" s="36"/>
+      <c r="A61" s="55"/>
       <c r="B61" s="6"/>
       <c r="E61" s="16"/>
-      <c r="F61" s="19"/>
-      <c r="G61" s="19"/>
-      <c r="H61" s="19"/>
-      <c r="I61" s="20"/>
+      <c r="F61" s="36"/>
+      <c r="G61" s="36"/>
+      <c r="H61" s="36"/>
+      <c r="I61" s="37"/>
     </row>
     <row r="62" spans="1:9" ht="9" customHeight="1">
-      <c r="A62" s="26" t="s">
+      <c r="A62" s="47" t="s">
         <v>63</v>
       </c>
-      <c r="B62" s="27"/>
-      <c r="C62" s="27"/>
-      <c r="D62" s="27"/>
-      <c r="E62" s="30" t="s">
+      <c r="B62" s="48"/>
+      <c r="C62" s="48"/>
+      <c r="D62" s="48"/>
+      <c r="E62" s="51" t="s">
         <v>64</v>
       </c>
-      <c r="F62" s="30"/>
-      <c r="G62" s="30"/>
-      <c r="H62" s="30"/>
-      <c r="I62" s="31"/>
+      <c r="F62" s="51"/>
+      <c r="G62" s="51"/>
+      <c r="H62" s="51"/>
+      <c r="I62" s="52"/>
     </row>
     <row r="63" spans="1:9" ht="9" customHeight="1">
-      <c r="A63" s="26"/>
-      <c r="B63" s="27"/>
-      <c r="C63" s="27"/>
-      <c r="D63" s="27"/>
-      <c r="E63" s="32" t="s">
+      <c r="A63" s="47"/>
+      <c r="B63" s="48"/>
+      <c r="C63" s="48"/>
+      <c r="D63" s="48"/>
+      <c r="E63" s="61" t="s">
+        <v>82</v>
+      </c>
+      <c r="F63" s="62"/>
+      <c r="G63" s="61" t="s">
         <v>65</v>
       </c>
-      <c r="F63" s="32"/>
-      <c r="G63" s="32"/>
-      <c r="H63" s="32"/>
+      <c r="H63" s="62"/>
       <c r="I63" s="4" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="64" spans="1:9" ht="9" customHeight="1">
-      <c r="A64" s="26"/>
-      <c r="B64" s="27"/>
-      <c r="C64" s="27"/>
-      <c r="D64" s="27"/>
-      <c r="E64" s="33"/>
-      <c r="F64" s="33"/>
-      <c r="G64" s="33"/>
-      <c r="H64" s="33"/>
+      <c r="A64" s="47"/>
+      <c r="B64" s="48"/>
+      <c r="C64" s="48"/>
+      <c r="D64" s="48"/>
+      <c r="E64" s="63"/>
+      <c r="F64" s="64"/>
+      <c r="G64" s="61"/>
+      <c r="H64" s="62"/>
       <c r="I64" s="4"/>
     </row>
     <row r="65" spans="1:9" ht="9" customHeight="1">
-      <c r="A65" s="26"/>
-      <c r="B65" s="27"/>
-      <c r="C65" s="27"/>
-      <c r="D65" s="27"/>
-      <c r="E65" s="33"/>
-      <c r="F65" s="33"/>
-      <c r="G65" s="33"/>
-      <c r="H65" s="33"/>
+      <c r="A65" s="47"/>
+      <c r="B65" s="48"/>
+      <c r="C65" s="48"/>
+      <c r="D65" s="48"/>
+      <c r="E65" s="63"/>
+      <c r="F65" s="64"/>
+      <c r="G65" s="61"/>
+      <c r="H65" s="62"/>
       <c r="I65" s="4"/>
     </row>
     <row r="66" spans="1:9" ht="9" customHeight="1">
-      <c r="A66" s="26"/>
-      <c r="B66" s="27"/>
-      <c r="C66" s="27"/>
-      <c r="D66" s="27"/>
-      <c r="E66" s="33"/>
-      <c r="F66" s="33"/>
-      <c r="G66" s="33"/>
-      <c r="H66" s="33"/>
+      <c r="A66" s="47"/>
+      <c r="B66" s="48"/>
+      <c r="C66" s="48"/>
+      <c r="D66" s="48"/>
+      <c r="E66" s="63"/>
+      <c r="F66" s="64"/>
+      <c r="G66" s="61"/>
+      <c r="H66" s="62"/>
       <c r="I66" s="14"/>
     </row>
     <row r="67" spans="1:9" ht="9" customHeight="1">
-      <c r="A67" s="26"/>
-      <c r="B67" s="27"/>
-      <c r="C67" s="27"/>
-      <c r="D67" s="27"/>
-      <c r="E67" s="33"/>
-      <c r="F67" s="33"/>
-      <c r="G67" s="33"/>
-      <c r="H67" s="33"/>
+      <c r="A67" s="47"/>
+      <c r="B67" s="48"/>
+      <c r="C67" s="48"/>
+      <c r="D67" s="48"/>
+      <c r="E67" s="63"/>
+      <c r="F67" s="64"/>
+      <c r="G67" s="61"/>
+      <c r="H67" s="62"/>
       <c r="I67" s="14"/>
     </row>
     <row r="68" spans="1:9" ht="9" customHeight="1">
-      <c r="A68" s="26"/>
-      <c r="B68" s="27"/>
-      <c r="C68" s="27"/>
-      <c r="D68" s="27"/>
-      <c r="E68" s="33"/>
-      <c r="F68" s="33"/>
-      <c r="G68" s="33"/>
-      <c r="H68" s="33"/>
+      <c r="A68" s="47"/>
+      <c r="B68" s="48"/>
+      <c r="C68" s="48"/>
+      <c r="D68" s="48"/>
+      <c r="E68" s="63"/>
+      <c r="F68" s="64"/>
+      <c r="G68" s="61"/>
+      <c r="H68" s="62"/>
       <c r="I68" s="14"/>
     </row>
     <row r="69" spans="1:9" ht="9" customHeight="1">
-      <c r="A69" s="26"/>
-      <c r="B69" s="27"/>
-      <c r="C69" s="27"/>
-      <c r="D69" s="27"/>
-      <c r="E69" s="33"/>
-      <c r="F69" s="33"/>
-      <c r="G69" s="33"/>
-      <c r="H69" s="33"/>
+      <c r="A69" s="47"/>
+      <c r="B69" s="48"/>
+      <c r="C69" s="48"/>
+      <c r="D69" s="48"/>
+      <c r="E69" s="63"/>
+      <c r="F69" s="64"/>
+      <c r="G69" s="61"/>
+      <c r="H69" s="62"/>
       <c r="I69" s="14"/>
     </row>
     <row r="70" spans="1:9" ht="9" customHeight="1">
-      <c r="A70" s="26"/>
-      <c r="B70" s="27"/>
-      <c r="C70" s="27"/>
-      <c r="D70" s="27"/>
-      <c r="E70" s="33"/>
-      <c r="F70" s="33"/>
-      <c r="G70" s="33"/>
-      <c r="H70" s="33"/>
+      <c r="A70" s="47"/>
+      <c r="B70" s="48"/>
+      <c r="C70" s="48"/>
+      <c r="D70" s="48"/>
+      <c r="E70" s="63"/>
+      <c r="F70" s="64"/>
+      <c r="G70" s="61"/>
+      <c r="H70" s="62"/>
       <c r="I70" s="14"/>
     </row>
     <row r="71" spans="1:9" ht="9" customHeight="1">
-      <c r="A71" s="26"/>
-      <c r="B71" s="27"/>
-      <c r="C71" s="27"/>
-      <c r="D71" s="27"/>
-      <c r="E71" s="33"/>
-      <c r="F71" s="33"/>
-      <c r="G71" s="33"/>
-      <c r="H71" s="33"/>
+      <c r="A71" s="47"/>
+      <c r="B71" s="48"/>
+      <c r="C71" s="48"/>
+      <c r="D71" s="48"/>
+      <c r="E71" s="63"/>
+      <c r="F71" s="64"/>
+      <c r="G71" s="61"/>
+      <c r="H71" s="62"/>
       <c r="I71" s="14"/>
     </row>
     <row r="72" spans="1:9" ht="9" customHeight="1">
-      <c r="A72" s="26"/>
-      <c r="B72" s="27"/>
-      <c r="C72" s="27"/>
-      <c r="D72" s="27"/>
-      <c r="E72" s="33"/>
-      <c r="F72" s="33"/>
-      <c r="G72" s="33"/>
-      <c r="H72" s="33"/>
+      <c r="A72" s="47"/>
+      <c r="B72" s="48"/>
+      <c r="C72" s="48"/>
+      <c r="D72" s="48"/>
+      <c r="E72" s="63"/>
+      <c r="F72" s="64"/>
+      <c r="G72" s="61"/>
+      <c r="H72" s="62"/>
       <c r="I72" s="14"/>
     </row>
     <row r="73" spans="1:9" ht="9" customHeight="1">
-      <c r="A73" s="26"/>
-      <c r="B73" s="27"/>
-      <c r="C73" s="27"/>
-      <c r="D73" s="27"/>
-      <c r="E73" s="33"/>
-      <c r="F73" s="33"/>
-      <c r="G73" s="33"/>
-      <c r="H73" s="33"/>
+      <c r="A73" s="47"/>
+      <c r="B73" s="48"/>
+      <c r="C73" s="48"/>
+      <c r="D73" s="48"/>
+      <c r="E73" s="63"/>
+      <c r="F73" s="64"/>
+      <c r="G73" s="61"/>
+      <c r="H73" s="62"/>
       <c r="I73" s="14"/>
     </row>
     <row r="74" spans="1:9" ht="9" customHeight="1">
-      <c r="A74" s="26"/>
-      <c r="B74" s="27"/>
-      <c r="C74" s="27"/>
-      <c r="D74" s="27"/>
-      <c r="E74" s="21" t="s">
+      <c r="A74" s="47"/>
+      <c r="B74" s="48"/>
+      <c r="C74" s="48"/>
+      <c r="D74" s="48"/>
+      <c r="E74" s="56" t="s">
         <v>67</v>
       </c>
-      <c r="F74" s="21"/>
-      <c r="G74" s="21"/>
-      <c r="H74" s="19"/>
-      <c r="I74" s="20"/>
+      <c r="F74" s="56"/>
+      <c r="G74" s="56"/>
+      <c r="H74" s="36"/>
+      <c r="I74" s="37"/>
     </row>
     <row r="75" spans="1:9" ht="9" customHeight="1">
-      <c r="A75" s="26"/>
-      <c r="B75" s="27"/>
-      <c r="C75" s="27"/>
-      <c r="D75" s="27"/>
-      <c r="E75" s="21" t="s">
+      <c r="A75" s="47"/>
+      <c r="B75" s="48"/>
+      <c r="C75" s="48"/>
+      <c r="D75" s="48"/>
+      <c r="E75" s="56" t="s">
         <v>68</v>
       </c>
-      <c r="F75" s="21"/>
-      <c r="G75" s="21"/>
-      <c r="H75" s="19"/>
-      <c r="I75" s="20"/>
+      <c r="F75" s="56"/>
+      <c r="G75" s="56"/>
+      <c r="H75" s="36"/>
+      <c r="I75" s="37"/>
     </row>
     <row r="76" spans="1:9" ht="9" customHeight="1">
-      <c r="A76" s="26"/>
-      <c r="B76" s="27"/>
-      <c r="C76" s="27"/>
-      <c r="D76" s="27"/>
-      <c r="E76" s="21" t="s">
+      <c r="A76" s="47"/>
+      <c r="B76" s="48"/>
+      <c r="C76" s="48"/>
+      <c r="D76" s="48"/>
+      <c r="E76" s="56" t="s">
         <v>69</v>
       </c>
-      <c r="F76" s="21"/>
-      <c r="G76" s="21"/>
-      <c r="H76" s="19"/>
-      <c r="I76" s="20"/>
+      <c r="F76" s="56"/>
+      <c r="G76" s="56"/>
+      <c r="H76" s="36"/>
+      <c r="I76" s="37"/>
     </row>
     <row r="77" spans="1:9" ht="9" customHeight="1">
-      <c r="A77" s="26"/>
-      <c r="B77" s="27"/>
-      <c r="C77" s="27"/>
-      <c r="D77" s="27"/>
-      <c r="E77" s="21" t="s">
+      <c r="A77" s="47"/>
+      <c r="B77" s="48"/>
+      <c r="C77" s="48"/>
+      <c r="D77" s="48"/>
+      <c r="E77" s="56" t="s">
         <v>70</v>
       </c>
-      <c r="F77" s="21"/>
-      <c r="G77" s="21"/>
-      <c r="H77" s="19"/>
-      <c r="I77" s="20"/>
+      <c r="F77" s="56"/>
+      <c r="G77" s="56"/>
+      <c r="H77" s="36"/>
+      <c r="I77" s="37"/>
     </row>
     <row r="78" spans="1:9" ht="9" customHeight="1">
-      <c r="A78" s="26"/>
-      <c r="B78" s="27"/>
-      <c r="C78" s="27"/>
-      <c r="D78" s="27"/>
-      <c r="E78" s="21" t="s">
+      <c r="A78" s="47"/>
+      <c r="B78" s="48"/>
+      <c r="C78" s="48"/>
+      <c r="D78" s="48"/>
+      <c r="E78" s="56" t="s">
         <v>71</v>
       </c>
-      <c r="F78" s="21"/>
-      <c r="G78" s="21"/>
-      <c r="H78" s="19"/>
-      <c r="I78" s="20"/>
+      <c r="F78" s="56"/>
+      <c r="G78" s="56"/>
+      <c r="H78" s="36"/>
+      <c r="I78" s="37"/>
     </row>
     <row r="79" spans="1:9" ht="9" customHeight="1" thickBot="1">
-      <c r="A79" s="28"/>
-      <c r="B79" s="29"/>
-      <c r="C79" s="29"/>
-      <c r="D79" s="29"/>
-      <c r="E79" s="25" t="s">
+      <c r="A79" s="49"/>
+      <c r="B79" s="50"/>
+      <c r="C79" s="50"/>
+      <c r="D79" s="50"/>
+      <c r="E79" s="60" t="s">
         <v>72</v>
       </c>
-      <c r="F79" s="25"/>
-      <c r="G79" s="25"/>
-      <c r="H79" s="23"/>
-      <c r="I79" s="24"/>
+      <c r="F79" s="60"/>
+      <c r="G79" s="60"/>
+      <c r="H79" s="58"/>
+      <c r="I79" s="59"/>
     </row>
     <row r="80" spans="1:9" ht="9" customHeight="1" thickTop="1">
-      <c r="G80" s="22" t="s">
+      <c r="G80" s="57" t="s">
         <v>73</v>
       </c>
-      <c r="H80" s="22"/>
-      <c r="I80" s="22"/>
+      <c r="H80" s="57"/>
+      <c r="I80" s="57"/>
     </row>
     <row r="81" customFormat="1" ht="9" customHeight="1"/>
     <row r="82" customFormat="1"/>
@@ -2368,34 +2382,74 @@
     <row r="87" customFormat="1"/>
     <row r="88" customFormat="1"/>
   </sheetData>
-  <mergeCells count="107">
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="G6:I6"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="D1:I1"/>
-    <mergeCell ref="D2:I2"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="G3:I3"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="F19:I19"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="F14:I14"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="F16:I16"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="E7:F7"/>
+  <mergeCells count="118">
+    <mergeCell ref="G80:I80"/>
+    <mergeCell ref="E76:G76"/>
+    <mergeCell ref="H76:I77"/>
+    <mergeCell ref="E77:G77"/>
+    <mergeCell ref="E78:G78"/>
+    <mergeCell ref="H78:I79"/>
+    <mergeCell ref="E79:G79"/>
+    <mergeCell ref="G63:H63"/>
+    <mergeCell ref="G64:H64"/>
+    <mergeCell ref="G65:H65"/>
+    <mergeCell ref="G66:H66"/>
+    <mergeCell ref="G67:H67"/>
+    <mergeCell ref="G68:H68"/>
+    <mergeCell ref="G69:H69"/>
+    <mergeCell ref="G70:H70"/>
+    <mergeCell ref="G71:H71"/>
+    <mergeCell ref="G72:H72"/>
+    <mergeCell ref="G73:H73"/>
+    <mergeCell ref="E63:F63"/>
+    <mergeCell ref="E64:F64"/>
+    <mergeCell ref="E65:F65"/>
+    <mergeCell ref="E66:F66"/>
+    <mergeCell ref="E67:F67"/>
+    <mergeCell ref="E68:F68"/>
+    <mergeCell ref="F61:I61"/>
+    <mergeCell ref="A62:D79"/>
+    <mergeCell ref="E62:I62"/>
+    <mergeCell ref="A51:A61"/>
+    <mergeCell ref="E74:G74"/>
+    <mergeCell ref="H74:I75"/>
+    <mergeCell ref="E75:G75"/>
+    <mergeCell ref="E69:F69"/>
+    <mergeCell ref="E70:F70"/>
+    <mergeCell ref="E71:F71"/>
+    <mergeCell ref="E72:F72"/>
+    <mergeCell ref="E73:F73"/>
+    <mergeCell ref="A40:A50"/>
+    <mergeCell ref="F40:I40"/>
+    <mergeCell ref="F41:I41"/>
+    <mergeCell ref="F42:I42"/>
+    <mergeCell ref="F43:I43"/>
+    <mergeCell ref="F44:I44"/>
+    <mergeCell ref="F45:I45"/>
+    <mergeCell ref="F60:I60"/>
+    <mergeCell ref="F46:I46"/>
+    <mergeCell ref="F47:I47"/>
+    <mergeCell ref="F48:I48"/>
+    <mergeCell ref="F49:I49"/>
+    <mergeCell ref="F50:I50"/>
+    <mergeCell ref="F51:I51"/>
+    <mergeCell ref="F52:I52"/>
+    <mergeCell ref="F53:I53"/>
+    <mergeCell ref="F54:I54"/>
+    <mergeCell ref="F55:I55"/>
+    <mergeCell ref="F56:I56"/>
+    <mergeCell ref="F57:I57"/>
+    <mergeCell ref="F58:I58"/>
+    <mergeCell ref="F59:I59"/>
+    <mergeCell ref="A33:A39"/>
+    <mergeCell ref="F33:I33"/>
+    <mergeCell ref="F34:I34"/>
+    <mergeCell ref="F39:I39"/>
+    <mergeCell ref="L34:M34"/>
+    <mergeCell ref="F35:I35"/>
+    <mergeCell ref="F36:I36"/>
+    <mergeCell ref="F37:I37"/>
+    <mergeCell ref="F38:I38"/>
     <mergeCell ref="L19:M19"/>
     <mergeCell ref="F20:I20"/>
     <mergeCell ref="L20:M20"/>
@@ -2420,62 +2474,33 @@
     <mergeCell ref="F30:I30"/>
     <mergeCell ref="F31:I31"/>
     <mergeCell ref="F32:I32"/>
-    <mergeCell ref="A33:A39"/>
-    <mergeCell ref="F33:I33"/>
-    <mergeCell ref="F34:I34"/>
-    <mergeCell ref="F39:I39"/>
-    <mergeCell ref="L34:M34"/>
-    <mergeCell ref="F35:I35"/>
-    <mergeCell ref="F36:I36"/>
-    <mergeCell ref="F37:I37"/>
-    <mergeCell ref="F38:I38"/>
-    <mergeCell ref="A40:A50"/>
-    <mergeCell ref="F40:I40"/>
-    <mergeCell ref="F41:I41"/>
-    <mergeCell ref="F42:I42"/>
-    <mergeCell ref="F43:I43"/>
-    <mergeCell ref="F44:I44"/>
-    <mergeCell ref="F45:I45"/>
-    <mergeCell ref="F60:I60"/>
-    <mergeCell ref="F46:I46"/>
-    <mergeCell ref="F47:I47"/>
-    <mergeCell ref="F48:I48"/>
-    <mergeCell ref="F49:I49"/>
-    <mergeCell ref="F50:I50"/>
-    <mergeCell ref="F51:I51"/>
-    <mergeCell ref="F52:I52"/>
-    <mergeCell ref="F53:I53"/>
-    <mergeCell ref="F54:I54"/>
-    <mergeCell ref="F55:I55"/>
-    <mergeCell ref="F56:I56"/>
-    <mergeCell ref="F57:I57"/>
-    <mergeCell ref="F58:I58"/>
-    <mergeCell ref="F59:I59"/>
-    <mergeCell ref="F61:I61"/>
-    <mergeCell ref="A62:D79"/>
-    <mergeCell ref="E62:I62"/>
-    <mergeCell ref="E63:H63"/>
-    <mergeCell ref="E64:H64"/>
-    <mergeCell ref="E65:H65"/>
-    <mergeCell ref="E66:H66"/>
-    <mergeCell ref="E67:H67"/>
-    <mergeCell ref="E68:H68"/>
-    <mergeCell ref="E69:H69"/>
-    <mergeCell ref="A51:A61"/>
-    <mergeCell ref="E70:H70"/>
-    <mergeCell ref="E71:H71"/>
-    <mergeCell ref="E72:H72"/>
-    <mergeCell ref="E73:H73"/>
-    <mergeCell ref="E74:G74"/>
-    <mergeCell ref="H74:I75"/>
-    <mergeCell ref="E75:G75"/>
-    <mergeCell ref="G80:I80"/>
-    <mergeCell ref="E76:G76"/>
-    <mergeCell ref="H76:I77"/>
-    <mergeCell ref="E77:G77"/>
-    <mergeCell ref="E78:G78"/>
-    <mergeCell ref="H78:I79"/>
-    <mergeCell ref="E79:G79"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="D1:I1"/>
+    <mergeCell ref="D2:I2"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="G6:I6"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.195138888888889" bottom="0" header="0" footer="0"/>

</xml_diff>

<commit_message>
feat: update maintenance templates for diesel engine, electric engine, electrical, motor pump, refrigerasi, sipil, and utility
</commit_message>
<xml_diff>
--- a/public/assets/templates/maintenance/diesel_engine.xlsx
+++ b/public/assets/templates/maintenance/diesel_engine.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\pt_bas\Engineering\public\assets\templates\maintenance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48B4B826-254D-475D-9091-72851F6DC0AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C3168FB-A544-4026-BCAD-9517DD7D336A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10560" xr2:uid="{197A4A4E-22CF-4E0D-A0A6-07FA889DE95B}"/>
   </bookViews>
@@ -237,18 +237,9 @@
     <t>Teknisi</t>
   </si>
   <si>
-    <t>Diketahui : Miftah Hasan Fuadi</t>
-  </si>
-  <si>
     <t>Staff Engineering</t>
   </si>
   <si>
-    <t>Diterima</t>
-  </si>
-  <si>
-    <t>Staff User</t>
-  </si>
-  <si>
     <t>FRM/EUT/01/009/014-02</t>
   </si>
   <si>
@@ -277,13 +268,22 @@
   </si>
   <si>
     <t>MID</t>
+  </si>
+  <si>
+    <t>Diperiksa : Miftah Hasan Fuadi</t>
+  </si>
+  <si>
+    <t>Diketahui : Reja Firmansyah</t>
+  </si>
+  <si>
+    <t>Supervisor Engineering</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -292,71 +292,78 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="8"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="8"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="7"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="12"/>
       <name val="Times New Roman"/>
-      <charset val="134"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="7"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="7"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="6"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="7"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -364,7 +371,7 @@
       <sz val="7"/>
       <color theme="1"/>
       <name val="Arial"/>
-      <charset val="134"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -381,7 +388,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -624,212 +631,283 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="69">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="19" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="22" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="21" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="2" xr:uid="{8D8AB921-6406-4838-8B6F-B9E269FE56FD}"/>
     <cellStyle name="Normal_Inspection Test Plan" xfId="1" xr:uid="{41E06106-563F-4589-AF04-89483409AEA5}"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1210,143 +1288,143 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" thickTop="1">
-      <c r="A1" s="23"/>
-      <c r="B1" s="24"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="27" t="s">
+      <c r="A1" s="44"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="28"/>
+      <c r="E1" s="48"/>
+      <c r="F1" s="48"/>
+      <c r="G1" s="48"/>
+      <c r="H1" s="48"/>
+      <c r="I1" s="49"/>
     </row>
     <row r="2" spans="1:9">
-      <c r="A2" s="25"/>
-      <c r="B2" s="26"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="29" t="s">
+      <c r="A2" s="46"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="50" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
-      <c r="H2" s="29"/>
-      <c r="I2" s="30"/>
+      <c r="E2" s="50"/>
+      <c r="F2" s="50"/>
+      <c r="G2" s="50"/>
+      <c r="H2" s="50"/>
+      <c r="I2" s="51"/>
     </row>
     <row r="3" spans="1:9" ht="10" customHeight="1">
       <c r="A3" s="1" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B3" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="31" t="s">
+      <c r="C3" s="57"/>
+      <c r="D3" s="57"/>
+      <c r="E3" s="52" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="32"/>
-      <c r="G3" s="33" t="s">
+      <c r="F3" s="53"/>
+      <c r="G3" s="54" t="s">
         <v>2</v>
       </c>
-      <c r="H3" s="34"/>
-      <c r="I3" s="35"/>
+      <c r="H3" s="55"/>
+      <c r="I3" s="56"/>
     </row>
     <row r="4" spans="1:9" ht="10" customHeight="1">
       <c r="A4" s="1" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B4" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20" t="s">
-        <v>80</v>
-      </c>
-      <c r="F4" s="20"/>
-      <c r="G4" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="H4" s="21"/>
-      <c r="I4" s="22"/>
+      <c r="C4" s="57"/>
+      <c r="D4" s="57"/>
+      <c r="E4" s="57" t="s">
+        <v>77</v>
+      </c>
+      <c r="F4" s="57"/>
+      <c r="G4" s="62" t="s">
+        <v>76</v>
+      </c>
+      <c r="H4" s="62"/>
+      <c r="I4" s="63"/>
     </row>
     <row r="5" spans="1:9" ht="10" customHeight="1">
       <c r="A5" s="1" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B5" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20" t="s">
-        <v>81</v>
-      </c>
-      <c r="F5" s="20"/>
-      <c r="G5" s="21" t="s">
+      <c r="C5" s="57"/>
+      <c r="D5" s="57"/>
+      <c r="E5" s="57" t="s">
+        <v>78</v>
+      </c>
+      <c r="F5" s="57"/>
+      <c r="G5" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="H5" s="21"/>
-      <c r="I5" s="22"/>
+      <c r="H5" s="62"/>
+      <c r="I5" s="63"/>
     </row>
     <row r="6" spans="1:9" ht="10" customHeight="1">
       <c r="A6" s="1" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B6" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="31" t="s">
+      <c r="C6" s="57"/>
+      <c r="D6" s="57"/>
+      <c r="E6" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="F6" s="32"/>
-      <c r="G6" s="21" t="s">
+      <c r="F6" s="53"/>
+      <c r="G6" s="62" t="s">
         <v>2</v>
       </c>
-      <c r="H6" s="21"/>
-      <c r="I6" s="22"/>
+      <c r="H6" s="62"/>
+      <c r="I6" s="63"/>
     </row>
     <row r="7" spans="1:9" ht="10" customHeight="1">
       <c r="A7" s="1" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B7" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="41"/>
-      <c r="F7" s="41"/>
-      <c r="G7" s="33"/>
-      <c r="H7" s="34"/>
-      <c r="I7" s="35"/>
+      <c r="C7" s="57"/>
+      <c r="D7" s="57"/>
+      <c r="E7" s="61"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="54"/>
+      <c r="H7" s="55"/>
+      <c r="I7" s="56"/>
     </row>
     <row r="8" spans="1:9" s="5" customFormat="1" ht="11" customHeight="1">
       <c r="A8" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B8" s="38" t="s">
+      <c r="B8" s="58" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="38"/>
-      <c r="D8" s="38"/>
+      <c r="C8" s="58"/>
+      <c r="D8" s="58"/>
       <c r="E8" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="F8" s="39" t="s">
+      <c r="F8" s="59" t="s">
         <v>8</v>
       </c>
-      <c r="G8" s="39"/>
-      <c r="H8" s="39"/>
-      <c r="I8" s="40"/>
+      <c r="G8" s="59"/>
+      <c r="H8" s="59"/>
+      <c r="I8" s="60"/>
     </row>
     <row r="9" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A9" s="44" t="s">
+      <c r="A9" s="39" t="s">
         <v>9</v>
       </c>
       <c r="B9" s="6"/>
@@ -1357,13 +1435,13 @@
         <v>11</v>
       </c>
       <c r="E9" s="16"/>
-      <c r="F9" s="36"/>
-      <c r="G9" s="36"/>
-      <c r="H9" s="36"/>
-      <c r="I9" s="37"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="22"/>
+      <c r="H9" s="22"/>
+      <c r="I9" s="23"/>
     </row>
     <row r="10" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A10" s="44"/>
+      <c r="A10" s="39"/>
       <c r="B10" s="6"/>
       <c r="C10" s="7" t="s">
         <v>10</v>
@@ -1372,13 +1450,13 @@
         <v>12</v>
       </c>
       <c r="E10" s="16"/>
-      <c r="F10" s="36"/>
-      <c r="G10" s="36"/>
-      <c r="H10" s="36"/>
-      <c r="I10" s="37"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="22"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="23"/>
     </row>
     <row r="11" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A11" s="44"/>
+      <c r="A11" s="39"/>
       <c r="B11" s="6"/>
       <c r="C11" s="7" t="s">
         <v>10</v>
@@ -1387,13 +1465,13 @@
         <v>13</v>
       </c>
       <c r="E11" s="16"/>
-      <c r="F11" s="36"/>
-      <c r="G11" s="36"/>
-      <c r="H11" s="36"/>
-      <c r="I11" s="37"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="22"/>
+      <c r="H11" s="22"/>
+      <c r="I11" s="23"/>
     </row>
     <row r="12" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A12" s="44"/>
+      <c r="A12" s="39"/>
       <c r="B12" s="6"/>
       <c r="C12" s="7" t="s">
         <v>10</v>
@@ -1402,13 +1480,13 @@
         <v>14</v>
       </c>
       <c r="E12" s="16"/>
-      <c r="F12" s="36"/>
-      <c r="G12" s="36"/>
-      <c r="H12" s="36"/>
-      <c r="I12" s="37"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="22"/>
+      <c r="H12" s="22"/>
+      <c r="I12" s="23"/>
     </row>
     <row r="13" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A13" s="44"/>
+      <c r="A13" s="39"/>
       <c r="B13" s="6"/>
       <c r="C13" s="7" t="s">
         <v>10</v>
@@ -1417,13 +1495,13 @@
         <v>15</v>
       </c>
       <c r="E13" s="16"/>
-      <c r="F13" s="36"/>
-      <c r="G13" s="36"/>
-      <c r="H13" s="36"/>
-      <c r="I13" s="37"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="22"/>
+      <c r="H13" s="22"/>
+      <c r="I13" s="23"/>
     </row>
     <row r="14" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A14" s="44"/>
+      <c r="A14" s="39"/>
       <c r="B14" s="6"/>
       <c r="C14" s="7" t="s">
         <v>10</v>
@@ -1432,13 +1510,13 @@
         <v>16</v>
       </c>
       <c r="E14" s="16"/>
-      <c r="F14" s="36"/>
-      <c r="G14" s="36"/>
-      <c r="H14" s="36"/>
-      <c r="I14" s="37"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="22"/>
+      <c r="H14" s="22"/>
+      <c r="I14" s="23"/>
     </row>
     <row r="15" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A15" s="44"/>
+      <c r="A15" s="39"/>
       <c r="B15" s="6"/>
       <c r="C15" s="7" t="s">
         <v>10</v>
@@ -1447,13 +1525,13 @@
         <v>17</v>
       </c>
       <c r="E15" s="16"/>
-      <c r="F15" s="36"/>
-      <c r="G15" s="36"/>
-      <c r="H15" s="36"/>
-      <c r="I15" s="37"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="22"/>
+      <c r="H15" s="22"/>
+      <c r="I15" s="23"/>
     </row>
     <row r="16" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A16" s="44"/>
+      <c r="A16" s="39"/>
       <c r="B16" s="6"/>
       <c r="C16" s="7" t="s">
         <v>10</v>
@@ -1462,13 +1540,13 @@
         <v>18</v>
       </c>
       <c r="E16" s="16"/>
-      <c r="F16" s="36"/>
-      <c r="G16" s="36"/>
-      <c r="H16" s="36"/>
-      <c r="I16" s="37"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="22"/>
+      <c r="H16" s="22"/>
+      <c r="I16" s="23"/>
     </row>
     <row r="17" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A17" s="44"/>
+      <c r="A17" s="39"/>
       <c r="B17" s="6"/>
       <c r="C17" s="7" t="s">
         <v>10</v>
@@ -1477,13 +1555,13 @@
         <v>19</v>
       </c>
       <c r="E17" s="16"/>
-      <c r="F17" s="36"/>
-      <c r="G17" s="36"/>
-      <c r="H17" s="36"/>
-      <c r="I17" s="37"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="22"/>
+      <c r="H17" s="22"/>
+      <c r="I17" s="23"/>
     </row>
     <row r="18" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A18" s="44"/>
+      <c r="A18" s="39"/>
       <c r="B18" s="6"/>
       <c r="C18" s="7" t="s">
         <v>10</v>
@@ -1492,13 +1570,13 @@
         <v>20</v>
       </c>
       <c r="E18" s="16"/>
-      <c r="F18" s="36"/>
-      <c r="G18" s="36"/>
-      <c r="H18" s="36"/>
-      <c r="I18" s="37"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="22"/>
+      <c r="H18" s="22"/>
+      <c r="I18" s="23"/>
     </row>
     <row r="19" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A19" s="44"/>
+      <c r="A19" s="39"/>
       <c r="B19" s="6"/>
       <c r="C19" s="7" t="s">
         <v>10</v>
@@ -1507,15 +1585,15 @@
         <v>21</v>
       </c>
       <c r="E19" s="16"/>
-      <c r="F19" s="36"/>
-      <c r="G19" s="36"/>
-      <c r="H19" s="36"/>
-      <c r="I19" s="37"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="22"/>
+      <c r="H19" s="22"/>
+      <c r="I19" s="23"/>
       <c r="L19" s="42"/>
       <c r="M19" s="42"/>
     </row>
     <row r="20" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A20" s="44"/>
+      <c r="A20" s="39"/>
       <c r="B20" s="6"/>
       <c r="C20" s="7" t="s">
         <v>10</v>
@@ -1524,15 +1602,15 @@
         <v>22</v>
       </c>
       <c r="E20" s="16"/>
-      <c r="F20" s="36"/>
-      <c r="G20" s="36"/>
-      <c r="H20" s="36"/>
-      <c r="I20" s="37"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="23"/>
       <c r="L20" s="43"/>
       <c r="M20" s="43"/>
     </row>
     <row r="21" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A21" s="44"/>
+      <c r="A21" s="39"/>
       <c r="B21" s="6"/>
       <c r="C21" s="7" t="s">
         <v>10</v>
@@ -1541,15 +1619,15 @@
         <v>23</v>
       </c>
       <c r="E21" s="16"/>
-      <c r="F21" s="36"/>
-      <c r="G21" s="36"/>
-      <c r="H21" s="36"/>
-      <c r="I21" s="37"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="22"/>
+      <c r="H21" s="22"/>
+      <c r="I21" s="23"/>
       <c r="L21" s="10"/>
       <c r="M21" s="10"/>
     </row>
     <row r="22" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A22" s="44"/>
+      <c r="A22" s="39"/>
       <c r="B22" s="6"/>
       <c r="C22" s="7" t="s">
         <v>10</v>
@@ -1558,15 +1636,15 @@
         <v>24</v>
       </c>
       <c r="E22" s="16"/>
-      <c r="F22" s="36"/>
-      <c r="G22" s="36"/>
-      <c r="H22" s="36"/>
-      <c r="I22" s="37"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="22"/>
+      <c r="H22" s="22"/>
+      <c r="I22" s="23"/>
       <c r="L22" s="10"/>
       <c r="M22" s="10"/>
     </row>
     <row r="23" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A23" s="44"/>
+      <c r="A23" s="39"/>
       <c r="B23" s="6"/>
       <c r="C23" s="7" t="s">
         <v>10</v>
@@ -1575,26 +1653,26 @@
         <v>25</v>
       </c>
       <c r="E23" s="16"/>
-      <c r="F23" s="36"/>
-      <c r="G23" s="36"/>
-      <c r="H23" s="36"/>
-      <c r="I23" s="37"/>
+      <c r="F23" s="22"/>
+      <c r="G23" s="22"/>
+      <c r="H23" s="22"/>
+      <c r="I23" s="23"/>
       <c r="L23" s="10"/>
       <c r="M23" s="10"/>
     </row>
     <row r="24" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A24" s="44"/>
+      <c r="A24" s="39"/>
       <c r="B24" s="6"/>
       <c r="E24" s="16"/>
-      <c r="F24" s="36"/>
-      <c r="G24" s="36"/>
-      <c r="H24" s="36"/>
-      <c r="I24" s="37"/>
+      <c r="F24" s="22"/>
+      <c r="G24" s="22"/>
+      <c r="H24" s="22"/>
+      <c r="I24" s="23"/>
       <c r="L24" s="43"/>
       <c r="M24" s="43"/>
     </row>
     <row r="25" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A25" s="44" t="s">
+      <c r="A25" s="39" t="s">
         <v>26</v>
       </c>
       <c r="B25" s="6"/>
@@ -1605,13 +1683,13 @@
         <v>27</v>
       </c>
       <c r="E25" s="16"/>
-      <c r="F25" s="36"/>
-      <c r="G25" s="36"/>
-      <c r="H25" s="36"/>
-      <c r="I25" s="37"/>
+      <c r="F25" s="22"/>
+      <c r="G25" s="22"/>
+      <c r="H25" s="22"/>
+      <c r="I25" s="23"/>
     </row>
     <row r="26" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A26" s="44"/>
+      <c r="A26" s="39"/>
       <c r="B26" s="6"/>
       <c r="C26" s="7" t="s">
         <v>10</v>
@@ -1620,13 +1698,13 @@
         <v>28</v>
       </c>
       <c r="E26" s="16"/>
-      <c r="F26" s="36"/>
-      <c r="G26" s="36"/>
-      <c r="H26" s="36"/>
-      <c r="I26" s="37"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="22"/>
+      <c r="H26" s="22"/>
+      <c r="I26" s="23"/>
     </row>
     <row r="27" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A27" s="44"/>
+      <c r="A27" s="39"/>
       <c r="B27" s="6"/>
       <c r="C27" s="7" t="s">
         <v>10</v>
@@ -1635,13 +1713,13 @@
         <v>29</v>
       </c>
       <c r="E27" s="16"/>
-      <c r="F27" s="36"/>
-      <c r="G27" s="36"/>
-      <c r="H27" s="36"/>
-      <c r="I27" s="37"/>
+      <c r="F27" s="22"/>
+      <c r="G27" s="22"/>
+      <c r="H27" s="22"/>
+      <c r="I27" s="23"/>
     </row>
     <row r="28" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A28" s="44"/>
+      <c r="A28" s="39"/>
       <c r="B28" s="6"/>
       <c r="C28" s="7" t="s">
         <v>10</v>
@@ -1650,15 +1728,15 @@
         <v>30</v>
       </c>
       <c r="E28" s="16"/>
-      <c r="F28" s="36"/>
-      <c r="G28" s="36"/>
-      <c r="H28" s="36"/>
-      <c r="I28" s="37"/>
-      <c r="L28" s="45"/>
-      <c r="M28" s="45"/>
+      <c r="F28" s="22"/>
+      <c r="G28" s="22"/>
+      <c r="H28" s="22"/>
+      <c r="I28" s="23"/>
+      <c r="L28" s="41"/>
+      <c r="M28" s="41"/>
     </row>
     <row r="29" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A29" s="44"/>
+      <c r="A29" s="39"/>
       <c r="B29" s="6"/>
       <c r="C29" s="7" t="s">
         <v>10</v>
@@ -1667,15 +1745,15 @@
         <v>31</v>
       </c>
       <c r="E29" s="16"/>
-      <c r="F29" s="36"/>
-      <c r="G29" s="36"/>
-      <c r="H29" s="36"/>
-      <c r="I29" s="37"/>
-      <c r="L29" s="45"/>
-      <c r="M29" s="45"/>
+      <c r="F29" s="22"/>
+      <c r="G29" s="22"/>
+      <c r="H29" s="22"/>
+      <c r="I29" s="23"/>
+      <c r="L29" s="41"/>
+      <c r="M29" s="41"/>
     </row>
     <row r="30" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A30" s="44"/>
+      <c r="A30" s="39"/>
       <c r="B30" s="6"/>
       <c r="C30" s="7" t="s">
         <v>10</v>
@@ -1684,15 +1762,15 @@
         <v>32</v>
       </c>
       <c r="E30" s="16"/>
-      <c r="F30" s="36"/>
-      <c r="G30" s="36"/>
-      <c r="H30" s="36"/>
-      <c r="I30" s="37"/>
+      <c r="F30" s="22"/>
+      <c r="G30" s="22"/>
+      <c r="H30" s="22"/>
+      <c r="I30" s="23"/>
       <c r="L30" s="11"/>
       <c r="M30" s="11"/>
     </row>
     <row r="31" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A31" s="44"/>
+      <c r="A31" s="39"/>
       <c r="B31" s="6"/>
       <c r="C31" s="7" t="s">
         <v>10</v>
@@ -1701,24 +1779,24 @@
         <v>33</v>
       </c>
       <c r="E31" s="16"/>
-      <c r="F31" s="36"/>
-      <c r="G31" s="36"/>
-      <c r="H31" s="36"/>
-      <c r="I31" s="37"/>
+      <c r="F31" s="22"/>
+      <c r="G31" s="22"/>
+      <c r="H31" s="22"/>
+      <c r="I31" s="23"/>
       <c r="L31" s="11"/>
       <c r="M31" s="11"/>
     </row>
     <row r="32" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A32" s="44"/>
+      <c r="A32" s="39"/>
       <c r="B32" s="6"/>
       <c r="E32" s="16"/>
-      <c r="F32" s="36"/>
-      <c r="G32" s="36"/>
-      <c r="H32" s="36"/>
-      <c r="I32" s="37"/>
+      <c r="F32" s="22"/>
+      <c r="G32" s="22"/>
+      <c r="H32" s="22"/>
+      <c r="I32" s="23"/>
     </row>
     <row r="33" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A33" s="46" t="s">
+      <c r="A33" s="40" t="s">
         <v>34</v>
       </c>
       <c r="B33" s="6"/>
@@ -1729,13 +1807,13 @@
         <v>35</v>
       </c>
       <c r="E33" s="16"/>
-      <c r="F33" s="36"/>
-      <c r="G33" s="36"/>
-      <c r="H33" s="36"/>
-      <c r="I33" s="37"/>
+      <c r="F33" s="22"/>
+      <c r="G33" s="22"/>
+      <c r="H33" s="22"/>
+      <c r="I33" s="23"/>
     </row>
     <row r="34" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A34" s="46"/>
+      <c r="A34" s="40"/>
       <c r="B34" s="6"/>
       <c r="C34" s="7" t="s">
         <v>10</v>
@@ -1744,15 +1822,15 @@
         <v>36</v>
       </c>
       <c r="E34" s="16"/>
-      <c r="F34" s="36"/>
-      <c r="G34" s="36"/>
-      <c r="H34" s="36"/>
-      <c r="I34" s="37"/>
-      <c r="L34" s="45"/>
-      <c r="M34" s="45"/>
+      <c r="F34" s="22"/>
+      <c r="G34" s="22"/>
+      <c r="H34" s="22"/>
+      <c r="I34" s="23"/>
+      <c r="L34" s="41"/>
+      <c r="M34" s="41"/>
     </row>
     <row r="35" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A35" s="46"/>
+      <c r="A35" s="40"/>
       <c r="B35" s="6"/>
       <c r="C35" s="7" t="s">
         <v>10</v>
@@ -1761,15 +1839,15 @@
         <v>37</v>
       </c>
       <c r="E35" s="16"/>
-      <c r="F35" s="36"/>
-      <c r="G35" s="36"/>
-      <c r="H35" s="36"/>
-      <c r="I35" s="37"/>
+      <c r="F35" s="22"/>
+      <c r="G35" s="22"/>
+      <c r="H35" s="22"/>
+      <c r="I35" s="23"/>
       <c r="L35" s="11"/>
       <c r="M35" s="11"/>
     </row>
     <row r="36" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A36" s="46"/>
+      <c r="A36" s="40"/>
       <c r="B36" s="6"/>
       <c r="C36" s="7" t="s">
         <v>10</v>
@@ -1778,15 +1856,15 @@
         <v>38</v>
       </c>
       <c r="E36" s="16"/>
-      <c r="F36" s="36"/>
-      <c r="G36" s="36"/>
-      <c r="H36" s="36"/>
-      <c r="I36" s="37"/>
+      <c r="F36" s="22"/>
+      <c r="G36" s="22"/>
+      <c r="H36" s="22"/>
+      <c r="I36" s="23"/>
       <c r="L36" s="11"/>
       <c r="M36" s="11"/>
     </row>
     <row r="37" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A37" s="46"/>
+      <c r="A37" s="40"/>
       <c r="B37" s="6"/>
       <c r="C37" s="7" t="s">
         <v>10</v>
@@ -1795,13 +1873,13 @@
         <v>39</v>
       </c>
       <c r="E37" s="16"/>
-      <c r="F37" s="36"/>
-      <c r="G37" s="36"/>
-      <c r="H37" s="36"/>
-      <c r="I37" s="37"/>
+      <c r="F37" s="22"/>
+      <c r="G37" s="22"/>
+      <c r="H37" s="22"/>
+      <c r="I37" s="23"/>
     </row>
     <row r="38" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A38" s="46"/>
+      <c r="A38" s="40"/>
       <c r="B38" s="6"/>
       <c r="C38" s="7" t="s">
         <v>10</v>
@@ -1810,22 +1888,22 @@
         <v>40</v>
       </c>
       <c r="E38" s="16"/>
-      <c r="F38" s="36"/>
-      <c r="G38" s="36"/>
-      <c r="H38" s="36"/>
-      <c r="I38" s="37"/>
+      <c r="F38" s="22"/>
+      <c r="G38" s="22"/>
+      <c r="H38" s="22"/>
+      <c r="I38" s="23"/>
     </row>
     <row r="39" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A39" s="46"/>
+      <c r="A39" s="40"/>
       <c r="B39" s="6"/>
       <c r="E39" s="16"/>
-      <c r="F39" s="36"/>
-      <c r="G39" s="36"/>
-      <c r="H39" s="36"/>
-      <c r="I39" s="37"/>
+      <c r="F39" s="22"/>
+      <c r="G39" s="22"/>
+      <c r="H39" s="22"/>
+      <c r="I39" s="23"/>
     </row>
     <row r="40" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A40" s="44" t="s">
+      <c r="A40" s="39" t="s">
         <v>41</v>
       </c>
       <c r="B40" s="6"/>
@@ -1836,13 +1914,13 @@
         <v>42</v>
       </c>
       <c r="E40" s="16"/>
-      <c r="F40" s="36"/>
-      <c r="G40" s="36"/>
-      <c r="H40" s="36"/>
-      <c r="I40" s="37"/>
+      <c r="F40" s="22"/>
+      <c r="G40" s="22"/>
+      <c r="H40" s="22"/>
+      <c r="I40" s="23"/>
     </row>
     <row r="41" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A41" s="44"/>
+      <c r="A41" s="39"/>
       <c r="B41" s="6"/>
       <c r="C41" s="7" t="s">
         <v>10</v>
@@ -1851,13 +1929,13 @@
         <v>43</v>
       </c>
       <c r="E41" s="16"/>
-      <c r="F41" s="36"/>
-      <c r="G41" s="36"/>
-      <c r="H41" s="36"/>
-      <c r="I41" s="37"/>
+      <c r="F41" s="22"/>
+      <c r="G41" s="22"/>
+      <c r="H41" s="22"/>
+      <c r="I41" s="23"/>
     </row>
     <row r="42" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A42" s="44"/>
+      <c r="A42" s="39"/>
       <c r="B42" s="6"/>
       <c r="C42" s="7" t="s">
         <v>10</v>
@@ -1866,13 +1944,13 @@
         <v>44</v>
       </c>
       <c r="E42" s="16"/>
-      <c r="F42" s="36"/>
-      <c r="G42" s="36"/>
-      <c r="H42" s="36"/>
-      <c r="I42" s="37"/>
+      <c r="F42" s="22"/>
+      <c r="G42" s="22"/>
+      <c r="H42" s="22"/>
+      <c r="I42" s="23"/>
     </row>
     <row r="43" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A43" s="44"/>
+      <c r="A43" s="39"/>
       <c r="B43" s="6"/>
       <c r="C43" s="7" t="s">
         <v>10</v>
@@ -1881,13 +1959,13 @@
         <v>45</v>
       </c>
       <c r="E43" s="16"/>
-      <c r="F43" s="36"/>
-      <c r="G43" s="36"/>
-      <c r="H43" s="36"/>
-      <c r="I43" s="37"/>
+      <c r="F43" s="22"/>
+      <c r="G43" s="22"/>
+      <c r="H43" s="22"/>
+      <c r="I43" s="23"/>
     </row>
     <row r="44" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A44" s="44"/>
+      <c r="A44" s="39"/>
       <c r="B44" s="6"/>
       <c r="C44" s="7" t="s">
         <v>10</v>
@@ -1896,13 +1974,13 @@
         <v>46</v>
       </c>
       <c r="E44" s="16"/>
-      <c r="F44" s="36"/>
-      <c r="G44" s="36"/>
-      <c r="H44" s="36"/>
-      <c r="I44" s="37"/>
+      <c r="F44" s="22"/>
+      <c r="G44" s="22"/>
+      <c r="H44" s="22"/>
+      <c r="I44" s="23"/>
     </row>
     <row r="45" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A45" s="44"/>
+      <c r="A45" s="39"/>
       <c r="B45" s="6"/>
       <c r="C45" s="7" t="s">
         <v>10</v>
@@ -1911,13 +1989,13 @@
         <v>47</v>
       </c>
       <c r="E45" s="16"/>
-      <c r="F45" s="36"/>
-      <c r="G45" s="36"/>
-      <c r="H45" s="36"/>
-      <c r="I45" s="37"/>
+      <c r="F45" s="22"/>
+      <c r="G45" s="22"/>
+      <c r="H45" s="22"/>
+      <c r="I45" s="23"/>
     </row>
     <row r="46" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A46" s="44"/>
+      <c r="A46" s="39"/>
       <c r="B46" s="6"/>
       <c r="C46" s="7" t="s">
         <v>10</v>
@@ -1926,13 +2004,13 @@
         <v>48</v>
       </c>
       <c r="E46" s="16"/>
-      <c r="F46" s="36"/>
-      <c r="G46" s="36"/>
-      <c r="H46" s="36"/>
-      <c r="I46" s="37"/>
+      <c r="F46" s="22"/>
+      <c r="G46" s="22"/>
+      <c r="H46" s="22"/>
+      <c r="I46" s="23"/>
     </row>
     <row r="47" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A47" s="44"/>
+      <c r="A47" s="39"/>
       <c r="B47" s="6"/>
       <c r="C47" s="7" t="s">
         <v>10</v>
@@ -1941,13 +2019,13 @@
         <v>49</v>
       </c>
       <c r="E47" s="17"/>
-      <c r="F47" s="36"/>
-      <c r="G47" s="36"/>
-      <c r="H47" s="36"/>
-      <c r="I47" s="37"/>
+      <c r="F47" s="22"/>
+      <c r="G47" s="22"/>
+      <c r="H47" s="22"/>
+      <c r="I47" s="23"/>
     </row>
     <row r="48" spans="1:13" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A48" s="44"/>
+      <c r="A48" s="39"/>
       <c r="B48" s="6"/>
       <c r="C48" s="7" t="s">
         <v>10</v>
@@ -1956,13 +2034,13 @@
         <v>50</v>
       </c>
       <c r="E48" s="17"/>
-      <c r="F48" s="36"/>
-      <c r="G48" s="36"/>
-      <c r="H48" s="36"/>
-      <c r="I48" s="37"/>
+      <c r="F48" s="22"/>
+      <c r="G48" s="22"/>
+      <c r="H48" s="22"/>
+      <c r="I48" s="23"/>
     </row>
     <row r="49" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A49" s="44"/>
+      <c r="A49" s="39"/>
       <c r="B49" s="6"/>
       <c r="C49" s="7" t="s">
         <v>10</v>
@@ -1971,22 +2049,22 @@
         <v>51</v>
       </c>
       <c r="E49" s="17"/>
-      <c r="F49" s="36"/>
-      <c r="G49" s="36"/>
-      <c r="H49" s="36"/>
-      <c r="I49" s="37"/>
+      <c r="F49" s="22"/>
+      <c r="G49" s="22"/>
+      <c r="H49" s="22"/>
+      <c r="I49" s="23"/>
     </row>
     <row r="50" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A50" s="44"/>
+      <c r="A50" s="39"/>
       <c r="B50" s="6"/>
       <c r="E50" s="16"/>
-      <c r="F50" s="36"/>
-      <c r="G50" s="36"/>
-      <c r="H50" s="36"/>
-      <c r="I50" s="37"/>
+      <c r="F50" s="22"/>
+      <c r="G50" s="22"/>
+      <c r="H50" s="22"/>
+      <c r="I50" s="23"/>
     </row>
     <row r="51" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A51" s="53" t="s">
+      <c r="A51" s="36" t="s">
         <v>52</v>
       </c>
       <c r="B51" s="6"/>
@@ -1997,13 +2075,13 @@
         <v>53</v>
       </c>
       <c r="E51" s="16"/>
-      <c r="F51" s="36"/>
-      <c r="G51" s="36"/>
-      <c r="H51" s="36"/>
-      <c r="I51" s="37"/>
+      <c r="F51" s="22"/>
+      <c r="G51" s="22"/>
+      <c r="H51" s="22"/>
+      <c r="I51" s="23"/>
     </row>
     <row r="52" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A52" s="54"/>
+      <c r="A52" s="37"/>
       <c r="B52" s="6"/>
       <c r="C52" s="7" t="s">
         <v>10</v>
@@ -2012,13 +2090,13 @@
         <v>54</v>
       </c>
       <c r="E52" s="16"/>
-      <c r="F52" s="36"/>
-      <c r="G52" s="36"/>
-      <c r="H52" s="36"/>
-      <c r="I52" s="37"/>
+      <c r="F52" s="22"/>
+      <c r="G52" s="22"/>
+      <c r="H52" s="22"/>
+      <c r="I52" s="23"/>
     </row>
     <row r="53" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A53" s="54"/>
+      <c r="A53" s="37"/>
       <c r="B53" s="6"/>
       <c r="C53" s="7" t="s">
         <v>10</v>
@@ -2027,13 +2105,13 @@
         <v>55</v>
       </c>
       <c r="E53" s="16"/>
-      <c r="F53" s="36"/>
-      <c r="G53" s="36"/>
-      <c r="H53" s="36"/>
-      <c r="I53" s="37"/>
+      <c r="F53" s="22"/>
+      <c r="G53" s="22"/>
+      <c r="H53" s="22"/>
+      <c r="I53" s="23"/>
     </row>
     <row r="54" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A54" s="54"/>
+      <c r="A54" s="37"/>
       <c r="B54" s="6"/>
       <c r="C54" s="7" t="s">
         <v>10</v>
@@ -2042,13 +2120,13 @@
         <v>56</v>
       </c>
       <c r="E54" s="16"/>
-      <c r="F54" s="36"/>
-      <c r="G54" s="36"/>
-      <c r="H54" s="36"/>
-      <c r="I54" s="37"/>
+      <c r="F54" s="22"/>
+      <c r="G54" s="22"/>
+      <c r="H54" s="22"/>
+      <c r="I54" s="23"/>
     </row>
     <row r="55" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A55" s="54"/>
+      <c r="A55" s="37"/>
       <c r="B55" s="6"/>
       <c r="C55" s="7" t="s">
         <v>10</v>
@@ -2057,13 +2135,13 @@
         <v>57</v>
       </c>
       <c r="E55" s="16"/>
-      <c r="F55" s="36"/>
-      <c r="G55" s="36"/>
-      <c r="H55" s="36"/>
-      <c r="I55" s="37"/>
+      <c r="F55" s="22"/>
+      <c r="G55" s="22"/>
+      <c r="H55" s="22"/>
+      <c r="I55" s="23"/>
     </row>
     <row r="56" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A56" s="54"/>
+      <c r="A56" s="37"/>
       <c r="B56" s="6"/>
       <c r="C56" s="7" t="s">
         <v>10</v>
@@ -2072,13 +2150,13 @@
         <v>58</v>
       </c>
       <c r="E56" s="16"/>
-      <c r="F56" s="36"/>
-      <c r="G56" s="36"/>
-      <c r="H56" s="36"/>
-      <c r="I56" s="37"/>
+      <c r="F56" s="22"/>
+      <c r="G56" s="22"/>
+      <c r="H56" s="22"/>
+      <c r="I56" s="23"/>
     </row>
     <row r="57" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A57" s="54"/>
+      <c r="A57" s="37"/>
       <c r="B57" s="6"/>
       <c r="C57" s="7" t="s">
         <v>10</v>
@@ -2087,13 +2165,13 @@
         <v>59</v>
       </c>
       <c r="E57" s="16"/>
-      <c r="F57" s="36"/>
-      <c r="G57" s="36"/>
-      <c r="H57" s="36"/>
-      <c r="I57" s="37"/>
+      <c r="F57" s="22"/>
+      <c r="G57" s="22"/>
+      <c r="H57" s="22"/>
+      <c r="I57" s="23"/>
     </row>
     <row r="58" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A58" s="54"/>
+      <c r="A58" s="37"/>
       <c r="B58" s="6"/>
       <c r="C58" s="7" t="s">
         <v>10</v>
@@ -2102,13 +2180,13 @@
         <v>60</v>
       </c>
       <c r="E58" s="16"/>
-      <c r="F58" s="36"/>
-      <c r="G58" s="36"/>
-      <c r="H58" s="36"/>
-      <c r="I58" s="37"/>
+      <c r="F58" s="22"/>
+      <c r="G58" s="22"/>
+      <c r="H58" s="22"/>
+      <c r="I58" s="23"/>
     </row>
     <row r="59" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A59" s="54"/>
+      <c r="A59" s="37"/>
       <c r="B59" s="6"/>
       <c r="C59" s="7" t="s">
         <v>10</v>
@@ -2117,13 +2195,13 @@
         <v>61</v>
       </c>
       <c r="E59" s="16"/>
-      <c r="F59" s="36"/>
-      <c r="G59" s="36"/>
-      <c r="H59" s="36"/>
-      <c r="I59" s="37"/>
+      <c r="F59" s="22"/>
+      <c r="G59" s="22"/>
+      <c r="H59" s="22"/>
+      <c r="I59" s="23"/>
     </row>
     <row r="60" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A60" s="54"/>
+      <c r="A60" s="37"/>
       <c r="B60" s="6"/>
       <c r="C60" s="7" t="s">
         <v>10</v>
@@ -2132,246 +2210,246 @@
         <v>62</v>
       </c>
       <c r="E60" s="16"/>
-      <c r="F60" s="36"/>
-      <c r="G60" s="36"/>
-      <c r="H60" s="36"/>
-      <c r="I60" s="37"/>
+      <c r="F60" s="22"/>
+      <c r="G60" s="22"/>
+      <c r="H60" s="22"/>
+      <c r="I60" s="23"/>
     </row>
     <row r="61" spans="1:9" s="9" customFormat="1" ht="9" customHeight="1">
-      <c r="A61" s="55"/>
+      <c r="A61" s="38"/>
       <c r="B61" s="6"/>
       <c r="E61" s="16"/>
-      <c r="F61" s="36"/>
-      <c r="G61" s="36"/>
-      <c r="H61" s="36"/>
-      <c r="I61" s="37"/>
+      <c r="F61" s="22"/>
+      <c r="G61" s="22"/>
+      <c r="H61" s="22"/>
+      <c r="I61" s="23"/>
     </row>
     <row r="62" spans="1:9" ht="9" customHeight="1">
-      <c r="A62" s="47" t="s">
+      <c r="A62" s="30" t="s">
         <v>63</v>
       </c>
-      <c r="B62" s="48"/>
-      <c r="C62" s="48"/>
-      <c r="D62" s="48"/>
-      <c r="E62" s="51" t="s">
+      <c r="B62" s="31"/>
+      <c r="C62" s="31"/>
+      <c r="D62" s="31"/>
+      <c r="E62" s="34" t="s">
         <v>64</v>
       </c>
-      <c r="F62" s="51"/>
-      <c r="G62" s="51"/>
-      <c r="H62" s="51"/>
-      <c r="I62" s="52"/>
+      <c r="F62" s="34"/>
+      <c r="G62" s="34"/>
+      <c r="H62" s="34"/>
+      <c r="I62" s="35"/>
     </row>
     <row r="63" spans="1:9" ht="9" customHeight="1">
-      <c r="A63" s="47"/>
-      <c r="B63" s="48"/>
-      <c r="C63" s="48"/>
-      <c r="D63" s="48"/>
-      <c r="E63" s="61" t="s">
-        <v>82</v>
-      </c>
-      <c r="F63" s="62"/>
-      <c r="G63" s="61" t="s">
+      <c r="A63" s="30"/>
+      <c r="B63" s="31"/>
+      <c r="C63" s="31"/>
+      <c r="D63" s="31"/>
+      <c r="E63" s="26" t="s">
+        <v>79</v>
+      </c>
+      <c r="F63" s="27"/>
+      <c r="G63" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="H63" s="62"/>
+      <c r="H63" s="27"/>
       <c r="I63" s="4" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="64" spans="1:9" ht="9" customHeight="1">
-      <c r="A64" s="47"/>
-      <c r="B64" s="48"/>
-      <c r="C64" s="48"/>
-      <c r="D64" s="48"/>
-      <c r="E64" s="63"/>
-      <c r="F64" s="64"/>
-      <c r="G64" s="61"/>
-      <c r="H64" s="62"/>
+      <c r="A64" s="30"/>
+      <c r="B64" s="31"/>
+      <c r="C64" s="31"/>
+      <c r="D64" s="31"/>
+      <c r="E64" s="28"/>
+      <c r="F64" s="29"/>
+      <c r="G64" s="26"/>
+      <c r="H64" s="27"/>
       <c r="I64" s="4"/>
     </row>
     <row r="65" spans="1:9" ht="9" customHeight="1">
-      <c r="A65" s="47"/>
-      <c r="B65" s="48"/>
-      <c r="C65" s="48"/>
-      <c r="D65" s="48"/>
-      <c r="E65" s="63"/>
-      <c r="F65" s="64"/>
-      <c r="G65" s="61"/>
-      <c r="H65" s="62"/>
+      <c r="A65" s="30"/>
+      <c r="B65" s="31"/>
+      <c r="C65" s="31"/>
+      <c r="D65" s="31"/>
+      <c r="E65" s="28"/>
+      <c r="F65" s="29"/>
+      <c r="G65" s="26"/>
+      <c r="H65" s="27"/>
       <c r="I65" s="4"/>
     </row>
     <row r="66" spans="1:9" ht="9" customHeight="1">
-      <c r="A66" s="47"/>
-      <c r="B66" s="48"/>
-      <c r="C66" s="48"/>
-      <c r="D66" s="48"/>
-      <c r="E66" s="63"/>
-      <c r="F66" s="64"/>
-      <c r="G66" s="61"/>
-      <c r="H66" s="62"/>
+      <c r="A66" s="30"/>
+      <c r="B66" s="31"/>
+      <c r="C66" s="31"/>
+      <c r="D66" s="31"/>
+      <c r="E66" s="28"/>
+      <c r="F66" s="29"/>
+      <c r="G66" s="26"/>
+      <c r="H66" s="27"/>
       <c r="I66" s="14"/>
     </row>
     <row r="67" spans="1:9" ht="9" customHeight="1">
-      <c r="A67" s="47"/>
-      <c r="B67" s="48"/>
-      <c r="C67" s="48"/>
-      <c r="D67" s="48"/>
-      <c r="E67" s="63"/>
-      <c r="F67" s="64"/>
-      <c r="G67" s="61"/>
-      <c r="H67" s="62"/>
+      <c r="A67" s="30"/>
+      <c r="B67" s="31"/>
+      <c r="C67" s="31"/>
+      <c r="D67" s="31"/>
+      <c r="E67" s="28"/>
+      <c r="F67" s="29"/>
+      <c r="G67" s="26"/>
+      <c r="H67" s="27"/>
       <c r="I67" s="14"/>
     </row>
     <row r="68" spans="1:9" ht="9" customHeight="1">
-      <c r="A68" s="47"/>
-      <c r="B68" s="48"/>
-      <c r="C68" s="48"/>
-      <c r="D68" s="48"/>
-      <c r="E68" s="63"/>
-      <c r="F68" s="64"/>
-      <c r="G68" s="61"/>
-      <c r="H68" s="62"/>
+      <c r="A68" s="30"/>
+      <c r="B68" s="31"/>
+      <c r="C68" s="31"/>
+      <c r="D68" s="31"/>
+      <c r="E68" s="28"/>
+      <c r="F68" s="29"/>
+      <c r="G68" s="26"/>
+      <c r="H68" s="27"/>
       <c r="I68" s="14"/>
     </row>
     <row r="69" spans="1:9" ht="9" customHeight="1">
-      <c r="A69" s="47"/>
-      <c r="B69" s="48"/>
-      <c r="C69" s="48"/>
-      <c r="D69" s="48"/>
-      <c r="E69" s="63"/>
-      <c r="F69" s="64"/>
-      <c r="G69" s="61"/>
-      <c r="H69" s="62"/>
+      <c r="A69" s="30"/>
+      <c r="B69" s="31"/>
+      <c r="C69" s="31"/>
+      <c r="D69" s="31"/>
+      <c r="E69" s="28"/>
+      <c r="F69" s="29"/>
+      <c r="G69" s="26"/>
+      <c r="H69" s="27"/>
       <c r="I69" s="14"/>
     </row>
     <row r="70" spans="1:9" ht="9" customHeight="1">
-      <c r="A70" s="47"/>
-      <c r="B70" s="48"/>
-      <c r="C70" s="48"/>
-      <c r="D70" s="48"/>
-      <c r="E70" s="63"/>
-      <c r="F70" s="64"/>
-      <c r="G70" s="61"/>
-      <c r="H70" s="62"/>
+      <c r="A70" s="30"/>
+      <c r="B70" s="31"/>
+      <c r="C70" s="31"/>
+      <c r="D70" s="31"/>
+      <c r="E70" s="28"/>
+      <c r="F70" s="29"/>
+      <c r="G70" s="26"/>
+      <c r="H70" s="27"/>
       <c r="I70" s="14"/>
     </row>
     <row r="71" spans="1:9" ht="9" customHeight="1">
-      <c r="A71" s="47"/>
-      <c r="B71" s="48"/>
-      <c r="C71" s="48"/>
-      <c r="D71" s="48"/>
-      <c r="E71" s="63"/>
-      <c r="F71" s="64"/>
-      <c r="G71" s="61"/>
-      <c r="H71" s="62"/>
+      <c r="A71" s="30"/>
+      <c r="B71" s="31"/>
+      <c r="C71" s="31"/>
+      <c r="D71" s="31"/>
+      <c r="E71" s="28"/>
+      <c r="F71" s="29"/>
+      <c r="G71" s="26"/>
+      <c r="H71" s="27"/>
       <c r="I71" s="14"/>
     </row>
     <row r="72" spans="1:9" ht="9" customHeight="1">
-      <c r="A72" s="47"/>
-      <c r="B72" s="48"/>
-      <c r="C72" s="48"/>
-      <c r="D72" s="48"/>
-      <c r="E72" s="63"/>
-      <c r="F72" s="64"/>
-      <c r="G72" s="61"/>
-      <c r="H72" s="62"/>
+      <c r="A72" s="30"/>
+      <c r="B72" s="31"/>
+      <c r="C72" s="31"/>
+      <c r="D72" s="31"/>
+      <c r="E72" s="28"/>
+      <c r="F72" s="29"/>
+      <c r="G72" s="26"/>
+      <c r="H72" s="27"/>
       <c r="I72" s="14"/>
     </row>
     <row r="73" spans="1:9" ht="9" customHeight="1">
-      <c r="A73" s="47"/>
-      <c r="B73" s="48"/>
-      <c r="C73" s="48"/>
-      <c r="D73" s="48"/>
-      <c r="E73" s="63"/>
-      <c r="F73" s="64"/>
-      <c r="G73" s="61"/>
-      <c r="H73" s="62"/>
+      <c r="A73" s="30"/>
+      <c r="B73" s="31"/>
+      <c r="C73" s="31"/>
+      <c r="D73" s="31"/>
+      <c r="E73" s="28"/>
+      <c r="F73" s="29"/>
+      <c r="G73" s="26"/>
+      <c r="H73" s="27"/>
       <c r="I73" s="14"/>
     </row>
     <row r="74" spans="1:9" ht="9" customHeight="1">
-      <c r="A74" s="47"/>
-      <c r="B74" s="48"/>
-      <c r="C74" s="48"/>
-      <c r="D74" s="48"/>
-      <c r="E74" s="56" t="s">
+      <c r="A74" s="30"/>
+      <c r="B74" s="31"/>
+      <c r="C74" s="31"/>
+      <c r="D74" s="31"/>
+      <c r="E74" s="21" t="s">
         <v>67</v>
       </c>
-      <c r="F74" s="56"/>
-      <c r="G74" s="56"/>
-      <c r="H74" s="36"/>
-      <c r="I74" s="37"/>
+      <c r="F74" s="21"/>
+      <c r="G74" s="21"/>
+      <c r="H74" s="22"/>
+      <c r="I74" s="23"/>
     </row>
     <row r="75" spans="1:9" ht="9" customHeight="1">
-      <c r="A75" s="47"/>
-      <c r="B75" s="48"/>
-      <c r="C75" s="48"/>
-      <c r="D75" s="48"/>
-      <c r="E75" s="56" t="s">
+      <c r="A75" s="30"/>
+      <c r="B75" s="31"/>
+      <c r="C75" s="31"/>
+      <c r="D75" s="31"/>
+      <c r="E75" s="21" t="s">
         <v>68</v>
       </c>
-      <c r="F75" s="56"/>
-      <c r="G75" s="56"/>
-      <c r="H75" s="36"/>
-      <c r="I75" s="37"/>
+      <c r="F75" s="21"/>
+      <c r="G75" s="21"/>
+      <c r="H75" s="22"/>
+      <c r="I75" s="23"/>
     </row>
     <row r="76" spans="1:9" ht="9" customHeight="1">
-      <c r="A76" s="47"/>
-      <c r="B76" s="48"/>
-      <c r="C76" s="48"/>
-      <c r="D76" s="48"/>
-      <c r="E76" s="56" t="s">
+      <c r="A76" s="30"/>
+      <c r="B76" s="31"/>
+      <c r="C76" s="31"/>
+      <c r="D76" s="31"/>
+      <c r="E76" s="64" t="s">
+        <v>80</v>
+      </c>
+      <c r="F76" s="64"/>
+      <c r="G76" s="64"/>
+      <c r="H76" s="22"/>
+      <c r="I76" s="23"/>
+    </row>
+    <row r="77" spans="1:9" ht="9" customHeight="1">
+      <c r="A77" s="30"/>
+      <c r="B77" s="31"/>
+      <c r="C77" s="31"/>
+      <c r="D77" s="31"/>
+      <c r="E77" s="21" t="s">
         <v>69</v>
       </c>
-      <c r="F76" s="56"/>
-      <c r="G76" s="56"/>
-      <c r="H76" s="36"/>
-      <c r="I76" s="37"/>
-    </row>
-    <row r="77" spans="1:9" ht="9" customHeight="1">
-      <c r="A77" s="47"/>
-      <c r="B77" s="48"/>
-      <c r="C77" s="48"/>
-      <c r="D77" s="48"/>
-      <c r="E77" s="56" t="s">
+      <c r="F77" s="21"/>
+      <c r="G77" s="21"/>
+      <c r="H77" s="22"/>
+      <c r="I77" s="23"/>
+    </row>
+    <row r="78" spans="1:9" ht="9" customHeight="1">
+      <c r="A78" s="30"/>
+      <c r="B78" s="31"/>
+      <c r="C78" s="31"/>
+      <c r="D78" s="31"/>
+      <c r="E78" s="66" t="s">
+        <v>81</v>
+      </c>
+      <c r="F78" s="66"/>
+      <c r="G78" s="66"/>
+      <c r="H78" s="22"/>
+      <c r="I78" s="23"/>
+    </row>
+    <row r="79" spans="1:9" ht="9" customHeight="1" thickBot="1">
+      <c r="A79" s="32"/>
+      <c r="B79" s="33"/>
+      <c r="C79" s="33"/>
+      <c r="D79" s="33"/>
+      <c r="E79" s="67" t="s">
+        <v>82</v>
+      </c>
+      <c r="F79" s="65"/>
+      <c r="G79" s="68"/>
+      <c r="H79" s="24"/>
+      <c r="I79" s="25"/>
+    </row>
+    <row r="80" spans="1:9" ht="9" customHeight="1" thickTop="1">
+      <c r="G80" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="F77" s="56"/>
-      <c r="G77" s="56"/>
-      <c r="H77" s="36"/>
-      <c r="I77" s="37"/>
-    </row>
-    <row r="78" spans="1:9" ht="9" customHeight="1">
-      <c r="A78" s="47"/>
-      <c r="B78" s="48"/>
-      <c r="C78" s="48"/>
-      <c r="D78" s="48"/>
-      <c r="E78" s="56" t="s">
-        <v>71</v>
-      </c>
-      <c r="F78" s="56"/>
-      <c r="G78" s="56"/>
-      <c r="H78" s="36"/>
-      <c r="I78" s="37"/>
-    </row>
-    <row r="79" spans="1:9" ht="9" customHeight="1" thickBot="1">
-      <c r="A79" s="49"/>
-      <c r="B79" s="50"/>
-      <c r="C79" s="50"/>
-      <c r="D79" s="50"/>
-      <c r="E79" s="60" t="s">
-        <v>72</v>
-      </c>
-      <c r="F79" s="60"/>
-      <c r="G79" s="60"/>
-      <c r="H79" s="58"/>
-      <c r="I79" s="59"/>
-    </row>
-    <row r="80" spans="1:9" ht="9" customHeight="1" thickTop="1">
-      <c r="G80" s="57" t="s">
-        <v>73</v>
-      </c>
-      <c r="H80" s="57"/>
-      <c r="I80" s="57"/>
+      <c r="H80" s="20"/>
+      <c r="I80" s="20"/>
     </row>
     <row r="81" customFormat="1" ht="9" customHeight="1"/>
     <row r="82" customFormat="1"/>
@@ -2383,73 +2461,36 @@
     <row r="88" customFormat="1"/>
   </sheetData>
   <mergeCells count="118">
-    <mergeCell ref="G80:I80"/>
+    <mergeCell ref="G4:I4"/>
+    <mergeCell ref="G5:I5"/>
+    <mergeCell ref="G6:I6"/>
     <mergeCell ref="E76:G76"/>
-    <mergeCell ref="H76:I77"/>
-    <mergeCell ref="E77:G77"/>
     <mergeCell ref="E78:G78"/>
-    <mergeCell ref="H78:I79"/>
     <mergeCell ref="E79:G79"/>
-    <mergeCell ref="G63:H63"/>
-    <mergeCell ref="G64:H64"/>
-    <mergeCell ref="G65:H65"/>
-    <mergeCell ref="G66:H66"/>
-    <mergeCell ref="G67:H67"/>
-    <mergeCell ref="G68:H68"/>
-    <mergeCell ref="G69:H69"/>
-    <mergeCell ref="G70:H70"/>
-    <mergeCell ref="G71:H71"/>
-    <mergeCell ref="G72:H72"/>
-    <mergeCell ref="G73:H73"/>
-    <mergeCell ref="E63:F63"/>
-    <mergeCell ref="E64:F64"/>
-    <mergeCell ref="E65:F65"/>
-    <mergeCell ref="E66:F66"/>
-    <mergeCell ref="E67:F67"/>
-    <mergeCell ref="E68:F68"/>
-    <mergeCell ref="F61:I61"/>
-    <mergeCell ref="A62:D79"/>
-    <mergeCell ref="E62:I62"/>
-    <mergeCell ref="A51:A61"/>
-    <mergeCell ref="E74:G74"/>
-    <mergeCell ref="H74:I75"/>
-    <mergeCell ref="E75:G75"/>
-    <mergeCell ref="E69:F69"/>
-    <mergeCell ref="E70:F70"/>
-    <mergeCell ref="E71:F71"/>
-    <mergeCell ref="E72:F72"/>
-    <mergeCell ref="E73:F73"/>
-    <mergeCell ref="A40:A50"/>
-    <mergeCell ref="F40:I40"/>
-    <mergeCell ref="F41:I41"/>
-    <mergeCell ref="F42:I42"/>
-    <mergeCell ref="F43:I43"/>
-    <mergeCell ref="F44:I44"/>
-    <mergeCell ref="F45:I45"/>
-    <mergeCell ref="F60:I60"/>
-    <mergeCell ref="F46:I46"/>
-    <mergeCell ref="F47:I47"/>
-    <mergeCell ref="F48:I48"/>
-    <mergeCell ref="F49:I49"/>
-    <mergeCell ref="F50:I50"/>
-    <mergeCell ref="F51:I51"/>
-    <mergeCell ref="F52:I52"/>
-    <mergeCell ref="F53:I53"/>
-    <mergeCell ref="F54:I54"/>
-    <mergeCell ref="F55:I55"/>
-    <mergeCell ref="F56:I56"/>
-    <mergeCell ref="F57:I57"/>
-    <mergeCell ref="F58:I58"/>
-    <mergeCell ref="F59:I59"/>
-    <mergeCell ref="A33:A39"/>
-    <mergeCell ref="F33:I33"/>
-    <mergeCell ref="F34:I34"/>
-    <mergeCell ref="F39:I39"/>
-    <mergeCell ref="L34:M34"/>
-    <mergeCell ref="F35:I35"/>
-    <mergeCell ref="F36:I36"/>
-    <mergeCell ref="F37:I37"/>
-    <mergeCell ref="F38:I38"/>
+    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="D1:I1"/>
+    <mergeCell ref="D2:I2"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="G3:I3"/>
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="F18:I18"/>
+    <mergeCell ref="F19:I19"/>
+    <mergeCell ref="E6:F6"/>
+    <mergeCell ref="G7:I7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="F15:I15"/>
+    <mergeCell ref="F16:I16"/>
+    <mergeCell ref="F17:I17"/>
+    <mergeCell ref="E7:F7"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="E5:F5"/>
     <mergeCell ref="L19:M19"/>
     <mergeCell ref="F20:I20"/>
     <mergeCell ref="L20:M20"/>
@@ -2474,33 +2515,70 @@
     <mergeCell ref="F30:I30"/>
     <mergeCell ref="F31:I31"/>
     <mergeCell ref="F32:I32"/>
-    <mergeCell ref="A1:C2"/>
-    <mergeCell ref="D1:I1"/>
-    <mergeCell ref="D2:I2"/>
-    <mergeCell ref="E3:F3"/>
-    <mergeCell ref="G3:I3"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="F18:I18"/>
-    <mergeCell ref="F19:I19"/>
-    <mergeCell ref="E6:F6"/>
-    <mergeCell ref="G7:I7"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="F13:I13"/>
-    <mergeCell ref="F14:I14"/>
-    <mergeCell ref="F15:I15"/>
-    <mergeCell ref="F16:I16"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="E7:F7"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="E4:F4"/>
-    <mergeCell ref="E5:F5"/>
-    <mergeCell ref="G4:I4"/>
-    <mergeCell ref="G5:I5"/>
-    <mergeCell ref="G6:I6"/>
+    <mergeCell ref="A33:A39"/>
+    <mergeCell ref="F33:I33"/>
+    <mergeCell ref="F34:I34"/>
+    <mergeCell ref="F39:I39"/>
+    <mergeCell ref="L34:M34"/>
+    <mergeCell ref="F35:I35"/>
+    <mergeCell ref="F36:I36"/>
+    <mergeCell ref="F37:I37"/>
+    <mergeCell ref="F38:I38"/>
+    <mergeCell ref="A40:A50"/>
+    <mergeCell ref="F40:I40"/>
+    <mergeCell ref="F41:I41"/>
+    <mergeCell ref="F42:I42"/>
+    <mergeCell ref="F43:I43"/>
+    <mergeCell ref="F44:I44"/>
+    <mergeCell ref="F45:I45"/>
+    <mergeCell ref="F60:I60"/>
+    <mergeCell ref="F46:I46"/>
+    <mergeCell ref="F47:I47"/>
+    <mergeCell ref="F48:I48"/>
+    <mergeCell ref="F49:I49"/>
+    <mergeCell ref="F50:I50"/>
+    <mergeCell ref="F51:I51"/>
+    <mergeCell ref="F52:I52"/>
+    <mergeCell ref="F53:I53"/>
+    <mergeCell ref="F54:I54"/>
+    <mergeCell ref="F55:I55"/>
+    <mergeCell ref="F56:I56"/>
+    <mergeCell ref="F57:I57"/>
+    <mergeCell ref="F58:I58"/>
+    <mergeCell ref="F59:I59"/>
+    <mergeCell ref="F61:I61"/>
+    <mergeCell ref="A62:D79"/>
+    <mergeCell ref="E62:I62"/>
+    <mergeCell ref="A51:A61"/>
+    <mergeCell ref="E74:G74"/>
+    <mergeCell ref="H74:I75"/>
+    <mergeCell ref="E75:G75"/>
+    <mergeCell ref="E69:F69"/>
+    <mergeCell ref="E70:F70"/>
+    <mergeCell ref="E71:F71"/>
+    <mergeCell ref="E72:F72"/>
+    <mergeCell ref="E73:F73"/>
+    <mergeCell ref="G80:I80"/>
+    <mergeCell ref="H76:I77"/>
+    <mergeCell ref="E77:G77"/>
+    <mergeCell ref="H78:I79"/>
+    <mergeCell ref="G63:H63"/>
+    <mergeCell ref="G64:H64"/>
+    <mergeCell ref="G65:H65"/>
+    <mergeCell ref="G66:H66"/>
+    <mergeCell ref="G67:H67"/>
+    <mergeCell ref="G68:H68"/>
+    <mergeCell ref="G69:H69"/>
+    <mergeCell ref="G70:H70"/>
+    <mergeCell ref="G71:H71"/>
+    <mergeCell ref="G72:H72"/>
+    <mergeCell ref="G73:H73"/>
+    <mergeCell ref="E63:F63"/>
+    <mergeCell ref="E64:F64"/>
+    <mergeCell ref="E65:F65"/>
+    <mergeCell ref="E66:F66"/>
+    <mergeCell ref="E67:F67"/>
+    <mergeCell ref="E68:F68"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0" right="0" top="0.195138888888889" bottom="0" header="0" footer="0"/>

</xml_diff>